<commit_message>
Add comprehensive article cleaning script with enhanced preprocessing steps
- Implemented a cleaning pipeline for the 'article' column in Excel and CSV files.
- Added steps for HTML entity decoding, script/style removal, HTML tag stripping, URL and email/IP address removal, emoji removal, and author byline/photo credit removal.
- Introduced source attribution removal to prevent data leakage.
- Normalized whitespace and collapsed consecutive blank lines.
- Included statistics reporting for rows changed and characters removed.
- Enhanced Excel writing functionality with improved formatting.
- Updated usage instructions for clarity.
</commit_message>
<xml_diff>
--- a/HF_cleaned.xlsx
+++ b/HF_cleaned.xlsx
@@ -907,7 +907,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>WALA na talagang kumabog sa The Amazing Praybeyt Benjamin bilang top-grosser sa nakaraang MMFF. Kumita ng P415-M sa takilya ang pelikulang ito nina Vice Ganda at Bimby Yap at nasa top 2 naman ang Feng Shui 2 nina Kris Aquino at Coco Martin kaya nagkaroon ng double thanksgiving party ang Star Cinema last weekend for their big success.</t>
+          <t>WALA na talagang kumabog sa The Amazing Praybeyt Benjamin bilang top-grosser sa nakaraang MMFF. Kumita ng P415-M sa takilya ang pelikulang ito nina Vice Ganda at Bim 2 naman ang Feng Shui 2 nina Kris Aquino at Coco Martin kaya nagkaroon ng double thanksgiving party ang Star Cinema last weekend for their big success.</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1432,7 +1432,7 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>ITINANGGI mismo ni Pangulong Duterte ang kumalat sa social media na siya ay pumanaw. "My reactions to my passing away.  I will ask God first if I... if He's available for interview kasi pupunta na ako 'dun. Ano mga mensahe ninyo? Dadalhin ko pari, obispo, lahat.  And yung last wish ng mga durugista, ilista ninyo.  Ako na ang magdala doon sa langin o sa impyerno.  Depende lang," sabi ni Duterte sa video na ipinost ng kanyang long-time partner na si Honelet Avancena, bagamat naka-pribado ang account nito. Matatandaang hindi nakadalo si Duterte sa pagtitipon sa Palo, Leyte noong Biyernes dahil sa masama ang kanyang pakiramdam. "For those who believe in the news that I passed away, then I request of you, please pray for me, for the eternal repose of my soul. Thank you," dagdag ni Duterte sa ikalawang video. Ipinost ni Avancena dalawang video ganap na alas-4 ng hapon.</t>
+          <t>ITINANGGI mismo ni Pangulong Duterte ang kumalat sa social media na siya ay pumanaw. "My reactions to my passing away. I will ask God first if I... if He's available for interview kasi pupunta na ako 'dun. Ano mga mensahe ninyo? Dadalhin ko pari, obispo, lahat. And yung last wish ng mga durugista, ilista ninyo. Ako na ang magdala doon sa langin o sa impyerno. Depende lang," sabi ni Duterte sa video na ipinost ng kanyang long-time partner na si Honelet Avancena, bagamat naka-pribado ang account nito. Matatandaang hindi nakadalo si Duterte sa pagtitipon sa Palo, Leyte noong Biyernes dahil sa masama ang kanyang pakiramdam. "For those who believe in the news that I passed away, then I request of you, please pray for me, for the eternal repose of my soul. Thank you," dagdag ni Duterte sa ikalawang video. Ipinost ni Avancena dalawang video ganap na alas-4 ng hapon.</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -2557,7 +2557,7 @@
       </c>
       <c r="B84" s="3" t="inlineStr">
         <is>
-          <t>PINAGBIGYAN ng Sandiganbayan First Division ang hiling ng kampo ni dating Sen. Ramon Bong Revilla Jr., na bigyan ito ng 20 araw upang magkomento sa petisyon ng prosekusyon na ipabalik sa kanya at kanyang mga kapwa akusado ang P124.5 milyong pondo na nawala sa gobyerno. Sa pagdinig, hiniling ni Atty. Estelito Mendoza, abugado ni Revilla, sa korte na bigyan sila ng 20 araw para makapaghain ng komento. Pinagbigyan ito ng korte at nag-utos na mayroong 10 araw ang prosekusyon para sagutin ang komento na ihahain ng kampo ni Revilla. Sa inihaing petisyon ng prosekusyon, sinabi nito na dapat maglabas ng utos ng korte at pabayaran na ang P124.5 milyong pondo ng gobyerno sa mga akusado kasama si Revilla. "[The decision was] based merely on reasonable doubt and not due to the absolute failure of the prosecution to prove his guilt," saad ng prosekusyon.  Nauna ng sinabi ng kampo ni Revilla na hindi ito dapat pagbayarin dahil siya ay pinawalang-sala ng korte sa kasong plunder. "Had the Court wanted to exclude Revilla, it could have simply and easily named Cambe and Napoles in the third paragraph, as it did in the first paragraph. It would not have used the collective term accused without exception and distinction," saad ng prosekusyon. Guilty ang hatol ng korte kay Janet Lim Napoles at Richard Cambe, dating aide ni Revilla.</t>
+          <t>PINAGBIGYAN ng Sandiganbayan First Division ang hiling ng kampo ni dating Sen. Ramon Bong Revilla Jr., na bigyan ito ng 20 araw upang magkomento sa petisyon ng prosekusyon na ipabalik sa kanya at kanyang mga kapwa akusado ang P124.5 milyong pondo na nawala sa gobyerno. Sa pagdinig, hiniling ni Atty. Estelito Mendoza, abugado ni Revilla, sa korte na bigyan sila ng 20 araw para makapaghain ng komento. Pinagbigyan ito ng korte at nag-utos na mayroong 10 araw ang prosekusyon para sagutin ang komento na ihahain ng kampo ni Revilla. Sa inihaing petisyon ng prosekusyon, sinabi nito na dapat maglabas ng utos ng korte at pabayaran na ang P124.5 milyong pondo ng gobyerno sa mga akusado kasama si Revilla. "[The decision was] based merely on reasonable doubt and not due to the absolute failure of the prosecution to prove his guilt," saad ng prosekusyon. Nauna ng sinabi ng kampo ni Revilla na hindi ito dapat pagbayarin dahil siya ay pinawalang-sala ng korte sa kasong plunder. "Had the Court wanted to exclude Revilla, it could have simply and easily named Cambe and Napoles in the third paragraph, as it did in the first paragraph. It would not have used the collective term accused without exception and distinction," saad ng prosekusyon. Guilty ang hatol ng korte kay Janet Lim Napoles at Richard Cambe, dating aide ni Revilla.</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
@@ -2657,7 +2657,7 @@
       </c>
       <c r="B88" s="3" t="inlineStr">
         <is>
-          <t>ARESTADO ang apat katao na nahulihan ng P3.5 milyong halaga ng shabu sa isang apartelle sa Quezon City kaninang ng umaga. Kinilala ang mga nahuli na sina Joshua Salazar ang kanyang tiyahin na si Mineya Amorine, Ruby Balani at Mary Jane Duran. Nagsagawa ng buybust operation ang pulisya laban sa mga suspek na nag-check in sa isang apartelle sa Araneta Ave., Brgy. Dona Imelda. Matapos makabili ang police poseur buyer ay pinasok na ng mga pulis ang kuwarto at nahuli ang mga suspek. Narekober sa mga suspek ang kalahating kilo ng shabu. Sa mga suspek umano kumukuha ng ipinagbabawal na gamot ang mga nagbebenta sa Maynila at mga karatig na probinsya. Ayon kay Salazar nautusan lamang siya ng isang Kristie upang dalhin ang isang plastic container kapalit ng P500.</t>
+          <t>ARESTADO ang apat katao na nahulihan ng P3.5 milyong halaga ng shabu sa isang apartelle sa Quezon City kaninang ng umaga. Kinilala ang mga nahuli na sina Joshua Salazar ang kanyang tiyahin na si Mineya Amorine, Ru uybust operation ang pulisya laban sa mga suspek na nag-check in sa isang apartelle sa Araneta Ave., Brgy. Dona Imelda. Matapos makabili ang police poseur buyer ay pinasok na ng mga pulis ang kuwarto at nahuli ang mga suspek. Narekober sa mga suspek ang kalahating kilo ng shabu. Sa mga suspek umano kumukuha ng ipinagbabawal na gamot ang mga nagbebenta sa Maynila at mga karatig na probinsya. Ayon kay Salazar nautusan lamang siya ng isang Kristie upang dalhin ang isang plastic container kapalit ng P500.</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
@@ -2782,7 +2782,7 @@
       </c>
       <c r="B93" s="3" t="inlineStr">
         <is>
-          <t>IGINIIT  ng Palasyo na sapat ang naging ayuda ng gobyerno sa 39-anyos na Pinay matapos na bitayin sa Saudi Arabi noong Martes dahil sa kasong murder. Sa isang briefing, nagpahatid din ng pakikiramay si Presidential Spokesperson at Chief Presidential Chief Legal Counsel Salvador Panelo sa pamilya ng nabitay na Pilipina.  "First, I would to express our condolences to the family, the bereaved family of the OFW that has been--who has been executed. Our government extended help to this Filipino, we provided lawyers or a lawyer for her and we gave regular updates to the family... ," sabi ni Panelo. Ayon sa Department of Foreign Affairs (DFA), ipinatupad ng mga otoridad ng Saudi ang parusang kamatayan laban sa Pinay matapos siyang mapatunayang guilty sa kasong murder. "It's just unfortunate that this particular case, the Sharia law does not apply where blood money can be a reason to stop the execution. So we condole with the family, but we tried... the DFA tried very hard to help," giit ni Panelo. (Bella Cariaso)</t>
+          <t>IGINIIT ng Palasyo na sapat ang naging ayuda ng gobyerno sa 39-anyos na Pinay matapos na bitayin sa Saudi Arabi noong Martes dahil sa kasong murder. Sa isang briefing, nagpahatid din ng pakikiramay si Presidential Spokesperson at Chief Presidential Chief Legal Counsel Salvador Panelo sa pamilya ng nabitay na Pilipina. "First, I would to express our condolences to the family, the bereaved family of the OFW that has been--who has been executed. Our government extended help to this Filipino, we provided lawyers or a lawyer for her and we gave regular updates to the family... ," sabi ni Panelo. Ayon sa Department of Foreign Affairs (DFA), ipinatupad ng mga otoridad ng Saudi ang parusang kamatayan laban sa Pinay matapos siyang mapatunayang guilty sa kasong murder. "It's just unfortunate that this particular case, the Sharia law does not apply where blood money can be a reason to stop the execution. So we condole with the family, but we tried... the DFA tried very hard to help," giit ni Panelo. (Bella Cariaso)</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
@@ -4232,7 +4232,7 @@
       </c>
       <c r="B151" s="3" t="inlineStr">
         <is>
-          <t>"I've been in this kind of situation many times in my previous fights. It doesn't scare me. I love being the underdog," ani Pacquiao, sa gitna ng mga ulat na ibinigay ng oddsmakers sa Las Vegas, ang pagdarausan ng kanilang laban sa Mayo 2, ang bentahe sa kanyang kalaban. "It even motivates me to train hard and go for the crown," ayon pa sa 36-anyos na boxer. Mukhang relaxed ang boxing champ at pupunta pa ito sa isa pa niyang trabaho, ang pagiging playing-coach ng Kia Carnival.	 "I will play on Wednesday," lahad ni Pacquiao sa ABS-CBN television. Ilang taon nang naghihintay ang boxing fans para sa laban sa pagitan ng dalawang boksingero, ang mga kinukonsiderang pinakamagaling na "pound-for-pound" na mga boksingero sa kanilang henerasyon. Makaraan ang ilang taong pagbabangayan at negosasyon, inanunsiyo nila noong Sabado na maghaharap sila sa isang laban na magpapaisa sa world welterweight crowns.	 Nag-umpisa na si Pacquiao sa kanyang light training para sa laban ilang linggo na ang nakararaan at nakitang tumatakbo na ng ilang laps at sumusuntok sa bag bilang paghahanda kay Mayweather. Kasunod ng mga ulat mula sa kampo ni Mayweather na pinupuna umano ang kanyang istilo sa paglaban, sinabi ni Pacquiao na malalaman ng American ang pagkakaiba ng panonood sa kanya sa screen at pagharap sa kanya sa ring. Ang 38-anyos na si Mayweather ay hindi pa natatalo sa loob ng 47 laban. Si Pacquiao ay mayroong 57 panalo at 5 talo, kabilang ang dalawang naranasan noong 2012. Kinumpira ng American promoter ni Pacquiao na si Bob arum na ang dalawang fighters ay hindi nagbigay ng anumang probisyon para sa rematch.</t>
+          <t>"I've been in this kind of situation many times in my previous fights. It doesn't scare me. I love being the underdog," ani Pacquiao, sa gitna ng mga ulat na ibinigay ng oddsmakers sa Las Vegas, ang pagdarausan ng kanilang laban sa Mayo 2, ang bentahe sa kanyang kalaban. "It even motivates me to train hard and go for the crown," ayon pa sa 36-anyos na boxer. Mukhang relaxed ang boxing champ at pupunta pa ito sa isa pa niyang trabaho, ang pagiging playing-coach ng Kia Carnival. "I will play on Wednesday," lahad ni Pacquiao sa ABS-CBN television. Ilang taon nang naghihintay ang boxing fans para sa laban sa pagitan ng dalawang boksingero, ang mga kinukonsiderang pinakamagaling na "pound-for-pound" na mga boksingero sa kanilang henerasyon. Makaraan ang ilang taong pagbabangayan at negosasyon, inanunsiyo nila noong Sabado na maghaharap sila sa isang laban na magpapaisa sa world welterweight crowns. Nag-umpisa na si Pacquiao sa kanyang light training para sa laban ilang linggo na ang nakararaan at nakitang tumatakbo na ng ilang laps at sumusuntok sa bag bilang paghahanda kay Mayweather. Kasunod ng mga ulat mula sa kampo ni Mayweather na pinupuna umano ang kanyang istilo sa paglaban, sinabi ni Pacquiao na malalaman ng American ang pagkakaiba ng panonood sa kanya sa screen at pagharap sa kanya sa ring. Ang 38-anyos na si Mayweather ay hindi pa natatalo sa loob ng 47 laban. Si Pacquiao ay mayroong 57 panalo at 5 talo, kabilang ang dalawang naranasan noong 2012. Kinumpira ng American promoter ni Pacquiao na si Bob arum na ang dalawang fighters ay hindi nagbigay ng anumang probisyon para sa rematch.</t>
         </is>
       </c>
       <c r="C151" s="2" t="inlineStr">
@@ -5382,7 +5382,7 @@
       </c>
       <c r="B197" s="3" t="inlineStr">
         <is>
-          <t>MULING ipinagtanggol ng Palasyo si Budget Secretary Benjamin Diokno matapos namang muling isnabin ang pagdinig sa Kamara.  "Secretary Benjamin Diokno has already manifested his position on the matter and his explanation for not attending the congressional hearing today is well-founded in fact and in law. We thus respect the Budget Secretary's decision and we are hopeful that knowledgeable men and women of Congress would similarly find the circumstances surrounding the said official's explanation justifiable as they perform their best in passing this year's budget," sabi Presidential Spokesperson at Chief Presidential Legal Counsel Salvador Panelo.  Tumanggi namang magkomento ang Palasyo sa panibagong alegasyon ng umano'y panunuhol ni Diokno na P40 bilyon sa Kamara.</t>
+          <t>MULING ipinagtanggol ng Palasyo si Budget Secretary Benjamin Diokno matapos namang muling isnabin ang pagdinig sa Kamara. "Secretary Benjamin Diokno has already manifested his position on the matter and his explanation for not attending the congressional hearing today is well-founded in fact and in law. We thus respect the Budget Secretary's decision and we are hopeful that knowledgeable men and women of Congress would similarly find the circumstances surrounding the said official's explanation justifiable as they perform their best in passing this year's budget," sabi Presidential Spokesperson at Chief Presidential Legal Counsel Salvador Panelo. Tumanggi namang magkomento ang Palasyo sa panibagong alegasyon ng umano'y panunuhol ni Diokno na P40 bilyon sa Kamara.</t>
         </is>
       </c>
       <c r="C197" s="2" t="inlineStr">
@@ -5957,7 +5957,7 @@
       </c>
       <c r="B220" s="3" t="inlineStr">
         <is>
-          <t>MAY isiningit na death penalty provision ang Kamara de Representantes sa mas mabigat na Dangerous Drugs law na inaprubahan nito sa ikatlo at huling pagbasa. Sa botong 172-0 at walang abstention, inaprubahan ng Kamara de Representantes ang House bill 8909. Ayon sa panukalang pagbabago sa Section 13 ng Comprehensive Dangerous Drugs Act ang sinumang mahuhuli na may dalang droga, gaano man karami, sa isang party, social gathering o meeting ang parusa ay habambuhay na pagkakabilanggo hanggang kamatayan.  Ito ay bukod pa sa P500,000 hanggang P10 milyong multa. Sa kasalukuyan ay walang parusang kamatayan sa bansa. May panukala na ibalik ang death penalty na naipasa na ang Kamara subalit hindi ito naaprubahan sa Senado. Isinama na rin sa mga maaaring maparusahan ang mga may-ari ng lugar kung saan may itinayong drug den.  Ang sinumang tao na malapit sa isang drug laboratory ay ituturing na sangkot sa paggawa ng ipinagbabawal na gamot. Sa ilalim ng panukala, kailangang sumailaim sa drug test ang mga atleta, propesyonal man o hindi, ng dalawang beses kada taon.</t>
+          <t>MAY isiningit na death penalty provision ang Kamara de Representantes sa mas mabigat na Dangerous Drugs law na inaprubahan nito sa ikatlo at huling pagbasa. Sa botong 172-0 at walang abstention, inaprubahan ng Kamara de Representantes ang House bill 8909. Ayon sa panukalang pagbabago sa Section 13 ng Comprehensive Dangerous Drugs Act ang sinumang mahuhuli na may dalang droga, gaano man karami, sa isang party, social gathering o meeting ang parusa ay habambuhay na pagkakabilanggo hanggang kamatayan. Ito ay bukod pa sa P500,000 hanggang P10 milyong multa. Sa kasalukuyan ay walang parusang kamatayan sa bansa. May panukala na ibalik ang death penalty na naipasa na ang Kamara subalit hindi ito naaprubahan sa Senado. Isinama na rin sa mga maaaring maparusahan ang mga may-ari ng lugar kung saan may itinayong drug den. Ang sinumang tao na malapit sa isang drug laboratory ay ituturing na sangkot sa paggawa ng ipinagbabawal na gamot. Sa ilalim ng panukala, kailangang sumailaim sa drug test ang mga atleta, propesyonal man o hindi, ng dalawang beses kada taon.</t>
         </is>
       </c>
       <c r="C220" s="2" t="inlineStr">
@@ -6532,7 +6532,7 @@
       </c>
       <c r="B243" s="3" t="inlineStr">
         <is>
-          <t>Ang karera ay tatawaging "The Tour for Heroes" na magsisimula sa Bataan kung saan ang lugar ay isang makasaysayan para sa mga Pilipinong sundalo na ibinuwis ang buhay laban sa pagkubkub ng Japanese forces sa World War II. "To start the 2015 Le Tour in Bataan at a time the nation is in mourning for the 44 slain SAF forces in Mamasapano [Maguindanao] inspires us to dedicate the race to our fallen heroes," saad ni Donna Lina Flavier, presidente ng race organizer na Ube Media Inc. "The Le Tour de Filipinas is not only about sports and competition, it's about fostering lasting peace among nations through cycling," dagdag ni Lina-Flavier. Isang panandaliang pananahimik ang iaalay sa mga nasawing SAF troopers (Fallen 44) sa pagbubukas ng makulay na seremonya kung saan si Bataan Gov. Abet Garcia at Balanga Mayor Joet Garcia ang magpapasinaya sa karera na iprinisinta ng Air21 at co-presented ng MVP sports Foundation at Smart. Mag-aalay din ng taimtim na pagdarasal ngayong umaga bago ang flag off para sa Balanga-Balanga 126-km Stage One ng International Cycling Union Asia Tour race na suportado rin ng Victory Liner, San Mig Zero, Novo Nordisk Pharmaceuticals Phils. at Canon kasama ang Isuzu, MAN Truck and Bus, Viking Rent-A-Car at NLEX bilang road partners. Mamumuno sa kampanya ng Pilipinas para sa 15-team race, ang 13 ay foreign squads, ay si defending champion Mark John Lexer Galedo ng PhilCycling's national men's team at Baler Ravina, ang 2012 winner para sa 7-Eleven by Road Bike Philippines. Batid nina Galedo at Ravina, at anim na iba pang Filipino riders na nakahanay sa mix, kung gaano kabigat ang labanan, partikular ang dalawang Iranian teams na pangungunahan ng dalawang mga dating kampeon at Asia's No. 1 sa UCI rankings. "We cannot promise anything but what is definite is that I and my teammates will do our best," saad ni Galedo na itinuon ang nagdaang dalawang taon, noong 2012 at 2014, na ang Le Tour ay pinagwagian ng Filipino kung saan ay walang nagpartisipang Iranian team.</t>
+          <t>Ang karera ay tatawaging "The Tour for Heroes" na magsisimula sa Bataan kung saan ang lugar ay isang makasaysayan para sa mga Pilipinong sundalo na ibinuwis ang buhay laban sa pagkubkub ng Japanese forces sa World War II. "To start the 2015 Le Tour in Bataan at a time the nation is in mourning for the 44 slain SAF forces in Mamasapano [Maguindanao] inspires us to dedicate the race to our fallen heroes," saad ni Donna Lina Flavier, presidente ng race organizer na Ube Media Inc. "The Le Tour de Filipinas is not only about sports and competition, it's about fostering lasting peace among nations through cycling," dagdag ni Lina-Flavier. Isang panandaliang pananahimik ang iaalay sa mga nasawing SAF troopers (Fallen 44) sa pagbubukas ng makulay na seremonya kung saan si Bataan Gov. Abet Garcia at Balanga Mayor Joet Garcia ang magpapasinaya sa karera na iprinisinta ng Air21 at co-presented ng MVP sports Foundation at Smart. Mag-aalay din ng taimtim na pagdarasal ngayong umaga bago ang flag off para sa Balanga-Balanga 126-km Stage One ng International Cycling Union Asia Tour race na suportado rin ng Victory Liner, San Mig Zero, Novo Nordisk Pharmaceuticals Phils. at Canon kasama ang Isuzu, MAN Truck and Bus, Viking Rent-A-Car at NLEX bilang road partners. Mamumuno sa kampanya ng Pilipinas para sa 15-team race, ang 13 ay foreign squads, ay si defending champion Mark John Lexer Galedo ng PhilCycling's national men's team at Baler Ravina, ang 2012 winner para sa 7-Eleven at Ravina, at anim na iba pang Filipino riders na nakahanay sa mix, kung gaano kabigat ang labanan, partikular ang dalawang Iranian teams na pangungunahan ng dalawang mga dating kampeon at Asia's No. 1 sa UCI rankings. "We cannot promise anything but what is definite is that I and my teammates will do our best," saad ni Galedo na itinuon ang nagdaang dalawang taon, noong 2012 at 2014, na ang Le Tour ay pinagwagian ng Filipino kung saan ay walang nagpartisipang Iranian team.</t>
         </is>
       </c>
       <c r="C243" s="2" t="inlineStr">
@@ -6857,7 +6857,7 @@
       </c>
       <c r="B256" s="3" t="inlineStr">
         <is>
-          <t>UMABOT na sa mahigit 4,000 kaso ng tigdas ang naitala, kabilang ang 70 nasawi sa nakalipas lamang na mahigit isang buwan, ayon sa Department of Health (DOH). Base sa datos mula sa DOH Epidemiology Bureau, mula Enero 1 hanggang Pebrero 9 ngayong taon, nakapagtala ang DOH ng 4,302 kaso ng tigdas na may 70 mga nasawi. Idinagdag ng DOH na  79 porsiyento sa mga nasawi ay may edad na isang buwan hanggang 31-anyos, at pawang hindi nagpabakuna. Samantalang ang edad naman ng mga apektado sa tigdas ay mula isang buwan hanggang 75-anyos, kung saan 34 porsiyento ay may edad na isa hanggang apat-anyos at 27 porsiyento sa mga kaso ay wala pang siyam-na-buwan. Sinabi pa ng DOH na 66 porsiyento ng mga apektaso ng tigdas ay pawang hindi nagpabakuna. Pinakamaraming kaso ng tigdas ang naitala sa National Capital Region na may 1,296 kaso at 18 nasawi, sinundan ng Calabarzon, na may 1,086 kaso at  25 na nasawi. Nakapagtala ang Central Luzon ng 481 kaso na may tatlong nasawi; Western Visayas, 212 kaso na may apat na nasawi; at sa Northern Mindanao, na may 189 kaso at limang nasawi. Nauna nang nagdeklara ang DOH ng measles outbreak sa Metro Manila, Central Luzon, Western at Eastern Visayas. "The causes of measles outbreak involved a number of factors or elements. Loss of public confidence and trust in vaccines in the immunization program brought about by the Dengvaxia controversy has been documented as one of many factors that contributed to vaccine hesitancy in the country," sabi ng DOH.</t>
+          <t>UMABOT na sa mahigit 4,000 kaso ng tigdas ang naitala, kabilang ang 70 nasawi sa nakalipas lamang na mahigit isang buwan, ayon sa Department of Health (DOH). Base sa datos mula sa DOH Epidemiology Bureau, mula Enero 1 hanggang Pebrero 9 ngayong taon, nakapagtala ang DOH ng 4,302 kaso ng tigdas na may 70 mga nasawi. Idinagdag ng DOH na 79 porsiyento sa mga nasawi ay may edad na isang buwan hanggang 31-anyos, at pawang hindi nagpabakuna. Samantalang ang edad naman ng mga apektado sa tigdas ay mula isang buwan hanggang 75-anyos, kung saan 34 porsiyento ay may edad na isa hanggang apat-anyos at 27 porsiyento sa mga kaso ay wala pang siyam-na-buwan. Sinabi pa ng DOH na 66 porsiyento ng mga apektaso ng tigdas ay pawang hindi nagpabakuna. Pinakamaraming kaso ng tigdas ang naitala sa National Capital Region na may 1,296 kaso at 18 nasawi, sinundan ng Calabarzon, na may 1,086 kaso at 25 na nasawi. Nakapagtala ang Central Luzon ng 481 kaso na may tatlong nasawi; Western Visayas, 212 kaso na may apat na nasawi; at sa Northern Mindanao, na may 189 kaso at limang nasawi. Nauna nang nagdeklara ang DOH ng measles outbreak sa Metro Manila, Central Luzon, Western at Eastern Visayas. "The causes of measles outbreak involved a number of factors or elements. Loss of public confidence and trust in vaccines in the immunization program brought about by the Dengvaxia controversy has been documented as one of many factors that contributed to vaccine hesitancy in the country," sabi ng DOH.</t>
         </is>
       </c>
       <c r="C256" s="2" t="inlineStr">
@@ -6882,7 +6882,7 @@
       </c>
       <c r="B257" s="3" t="inlineStr">
         <is>
-          <t>Kabilang sa mga reporma ngayong taon ang mas mabilis at mas maginhawang pakikipagtransaksiyon sa BOC, mas mahusay na koleksiyon ng buwis, at isang pinaigting na kampanya laban sa smuggling. Ang pinakamahalaga sa mga ito ay ang modernisasyon at automation ng mga serbisyo na nakaangkla sa pagpapatupad ng updated e-commerce technology bilang paghahanda sa paglulunsad ng ASEAN Economic Community. Sa Hunyo 2015, ang BOC, sa pamumuno ni Commissioner John Philip P. Sevilla, ay tinatanaw ang katuparan ng mga sumusunod na programa: fully electronic, paperless bureau; single, centralized assessment service; single, centralized valuation database; sale or disposition ng mga produktong inabandona, kinumpiska o isinuko bilang penalty sa loob ng dalawang buwan matapos ibaba ng resolusyon ng legal proceedings; at full electronic record-keeping para sa Customs-bonded na mga warehouse. Magiging katuwang ito ng limang taon na Strategic Plan (2013-2017), na isang action-oriented initiative upang gawing mahusay ang administrasyon ng Customs sa pamamagitan ng goal-setting at resource allocation hanggang 2017. Mayroong open engagement ang BOC sa pribadong seKtor sa pagbabalangkas ng mga polisiya, kung saan ginagawa ang karamihan ng mga aktibidad sa pakikipagkonsulta sa aktibong partisipasyon ng mga partner nito. Ang isang katanggap-tanggap na BOC project ay ang online tracking system (www.customs.gov.ph) na inilusad noong Disyembre 2014, kung saan maaaring makita ng mga tatanggap at nagpadala ng mga balikbayan box ang status nito. Laman ng tracker ang listahan ng lahat ng balikbayan box shipment na tangan ng mga lokal na cargo forwarder sa Customs, ang bansang pinanggalingan nito, ang papasukang daungan nito sa Pilipinas, at ang bills of lading na may bilang ng mga shipment.</t>
+          <t>Kabilang sa mga reporma ngayong taon ang mas mabilis at mas maginhawang pakikipagtransaksiyon sa BOC, mas mahusay na koleksiyon ng buwis, at isang pinaigting na kampanya laban sa smuggling. Ang pinakamahalaga sa mga ito ay ang modernisasyon at automation ng mga serbisyo na nakaangkla sa pagpapatupad ng updated e-commerce technology bilang paghahanda sa paglulunsad ng ASEAN Economic Community. Sa Hunyo 2015, ang BOC, sa pamumuno ni Commissioner John Philip P. Sevilla, ay tinatanaw ang katuparan ng mga sumusunod na programa: fully electronic, paperless bureau; single, centralized assessment service; single, centralized valuation database; sale or disposition ng mga produktong inabandona, kinumpiska o isinuko bilang penalty sa loob ng dalawang buwan matapos ibaba ng resolusyon ng legal proceedings; at full electronic record-keeping para sa Customs-bonded na mga warehouse. Magiging katuwang ito ng limang taon na Strategic Plan (2013-2017), na isang action-oriented initiative upang gawing mahusay ang administrasyon ng Customs sa pamamagitan ng goal-setting at resource allocation hanggang 2017. Mayroong open engagement ang BOC sa pribadong seKtor sa pagbabalangkas ng mga polisiya, kung saan ginagawa ang karamihan ng mga aktibidad sa pakikipagkonsulta sa aktibong partisipasyon ng mga partner nito. Ang isang katanggap-tanggap na BOC project ay ang online tracking system ( na inilusad noong Disyembre 2014, kung saan maaaring makita ng mga tatanggap at nagpadala ng mga balikbayan box ang status nito. Laman ng tracker ang listahan ng lahat ng balikbayan box shipment na tangan ng mga lokal na cargo forwarder sa Customs, ang bansang pinanggalingan nito, ang papasukang daungan nito sa Pilipinas, at ang bills of lading na may bilang ng mga shipment.</t>
         </is>
       </c>
       <c r="C257" s="2" t="inlineStr">
@@ -6982,7 +6982,7 @@
       </c>
       <c r="B261" s="3" t="inlineStr">
         <is>
-          <t>"The PNP-SAF's operation in Mamasapano was doomed to fail, and the fault lies squarely with Aquino," pahayag ni Labog. Sinabi ni Labog na tinangka ni Aquino na ilihis ang kanyang pananagutan sa operasyon sa pag-aresto sa dalawang international terrorist na sina Zulkifli bin Hir alias "Marwan," at Basit Usman nang tumanggi itong sagutin ang katanungan kung sino ang nag-apruba sa misyon ng PNP-SAF matapos ang kanyang talumpati sa telebisyon noong Miyerkules. "This was belied by Chief Supt. Getulio Napenas, the sacked commander of the SAF, who claimed that the chief executive had knowledge of the operation," ani Labog. Samantala, iminungkahi rin ni University of the Philippines (UP) Prof. Clarita Carlos, na nagsilbi bilang pangulo ng National Defense College of the Philippines (NDCP), ang pagbibitiw ni Interior and Local Government Secretary Mar Roxas sa puwesto matapos niyang aminin na wala siyang alam sa ikinasang operasyon ng PNP-SAF. "Kung ako si Mar Roxas, magre-resign ako. Bakit ang dami mong hindi alam? Kung meron ka pang respeto sa sarili mo, mag-resign ka kasi mukhang mayroong ibang gumagalaw at iba 'yung namamahala, nakikialam d'yan sa PNP," ayon kay Carlos.</t>
+          <t>"The PNP-SAF's operation in Mamasapano was doomed to fail, and the fault lies squarely with Aquino," pahayag ni Labog. Sinabi ni Labog na tinangka ni Aquino na ilihis ang kanyang pananagutan sa operasyon sa pag-aresto sa dalawang international terrorist na sina Zulkifli bin Hir alias "Marwan," at Basit Usman nang tumanggi itong sagutin ang katanungan kung sino ang nag-apruba sa misyon ng PNP-SAF matapos ang kanyang talumpati sa telebisyon noong Miyerkules. "This was belied , the sacked commander of the SAF, who claimed that the chief executive had knowledge of the operation," ani Labog. Samantala, iminungkahi rin ni University of the Philippines (UP) Prof. Clarita Carlos, na nagsilbi bilang pangulo ng National Defense College of the Philippines (NDCP), ang pagbibitiw ni Interior and Local Government Secretary Mar Roxas sa puwesto matapos niyang aminin na wala siyang alam sa ikinasang operasyon ng PNP-SAF. "Kung ako si Mar Roxas, magre-resign ako. Bakit ang dami mong hindi alam? Kung meron ka pang respeto sa sarili mo, mag-resign ka kasi mukhang mayroong ibang gumagalaw at iba 'yung namamahala, nakikialam d'yan sa PNP," ayon kay Carlos.</t>
         </is>
       </c>
       <c r="C261" s="2" t="inlineStr">
@@ -7232,7 +7232,7 @@
       </c>
       <c r="B271" s="3" t="inlineStr">
         <is>
-          <t>ILANG shooting days na lang, matatapos na ang MMFF entry ng Star Cinema starring Vice Ganda, Richard Yap at Bimby Yap na The Amazing: Praybeyt Benjamin na nagpresscon na kahapon. Kung ganado sa shooting si Vice, mas ganado si Sir Chief kaya nakapag-comment ang una na ang galing-galing ni Richard sa nasabing movie.</t>
+          <t>ILANG shooting days na lang, matatapos na ang MMFF entry ng Star Cinema starring Vice Ganda, Richard Yap at Bim : Praybeyt Benjamin na nagpresscon na kahapon. Kung ganado sa shooting si Vice, mas ganado si Sir Chief kaya nakapag-comment ang una na ang galing-galing ni Richard sa nasabing movie.</t>
         </is>
       </c>
       <c r="C271" s="2" t="inlineStr">
@@ -10257,7 +10257,7 @@
       </c>
       <c r="B392" s="3" t="inlineStr">
         <is>
-          <t>TATLO ang patay, samantalang anim na iba pa ang nasugatan, kabilang ang dalawang pulis matapos ang pamamaril sa Teresa, Rizal Huwebes ng gabi. Sa ulat mula sa Rizal Provincial Police Office, sinabi nito na nasa harap ng kanyang bahay ang biktimang si Ruben Francisco nang bigla na lamang siyang barilin ng isang John Albert Araojo. Sumunod na binaril ni Araojo si Wildredo Lukban na nasa bisinidad at isang Celso Bernales Jr., isang tricycle driver na naghihintay ng pasahero nang mangyari ang insidente, ayon sa pulisya. Dead on the spot ang tatlong biktima, ayon kay Senior Insp. Marinell Fronda, chief ng Teresa Municipal Police Station.  Rumesponde sina Police Officer 3 Emillano Pantaleon at  Police Officer 1 Eleuterio Mina ngunit pinaputukan din ng suspek. Apat pang iba pa ang nasugatan sa pamamaril, ayon sa pulisya.  Idinagdag ng pulisya na gumanti ng putok ang mga pulis bagamat nagawang makatakas patungong munisipalidad ng  Morong sakay ng kanyang motorsiklo. Nagsasagawa na ng manhunt lanan sa suspek. Dinala ang mga biktima sa Saint Therese Hospital para magamot. Inaalam pa ng pulisya ang motibo ng pamamaril.</t>
+          <t>TATLO ang patay, samantalang anim na iba pa ang nasugatan, kabilang ang dalawang pulis matapos ang pamamaril sa Teresa, Rizal Huwebes ng gabi. Sa ulat mula sa Rizal Provincial Police Office, sinabi nito na nasa harap ng kanyang bahay ang biktimang si Ruben Francisco nang bigla na lamang siyang barilin ng isang John Albert Araojo. Sumunod na binaril ni Araojo si Wildredo Lukban na nasa bisinidad at isang Celso Bernales Jr., isang tricycle driver na naghihintay ng pasahero nang mangyari ang insidente, ayon sa pulisya. Dead on the spot ang tatlong biktima, ayon kay Senior Insp. Marinell Fronda, chief ng Teresa Municipal Police Station. Rumesponde sina Police Officer 3 Emillano Pantaleon at Police Officer 1 Eleuterio Mina ngunit pinaputukan din ng suspek. Apat pang iba pa ang nasugatan sa pamamaril, ayon sa pulisya. Idinagdag ng pulisya na gumanti ng putok ang mga pulis bagamat nagawang makatakas patungong munisipalidad ng Morong sakay ng kanyang motorsiklo. Nagsasagawa na ng manhunt lanan sa suspek. Dinala ang mga biktima sa Saint Therese Hospital para magamot. Inaalam pa ng pulisya ang motibo ng pamamaril.</t>
         </is>
       </c>
       <c r="C392" s="2" t="inlineStr">
@@ -12132,7 +12132,7 @@
       </c>
       <c r="B467" s="3" t="inlineStr">
         <is>
-          <t>Ibinahagi ni Alden kung gaano kasaya at ka-challenging na makatrabaho ang superstar. "Siya 'yung epitome ng perfect acting, eh. Natural na natural. Alam mo na 'yung mga words na ginagamit niya ay galing sa puso talaga. Sobrang nag-enjoy talaga ako na nakatrabaho ko siya at mas lalong nadagdagan ang self-confidence ko dahil nagkaroon ako ng pagkakataon na makatrabaho ang nag-iisang superstar." Proud siya na kinatawan niya ang bansa sa nasabing international film festival. "It's such a blessing to experience attending this film festival. I was able to meet the stars and directors from different countries at paniguradong isa ito sa highlights ng aking career bilang isang aktor. The experience inspires me to do more and be the best that I can be." Samantala, napansin naman ng isang Vietnamese entertainment website na www.ngoisao.net si Alden at tinawag pa nila itong "Dien vien noi tieng cua" o sa Ingles ay Philippines' Famous Actor.</t>
+          <t>Ibinahagi ni Alden kung gaano kasaya at ka-challenging na makatrabaho ang superstar. "Siya 'yung epitome ng perfect acting, eh. Natural na natural. Alam mo na 'yung mga words na ginagamit niya ay galing sa puso talaga. Sobrang nag-enjoy talaga ako na nakatrabaho ko siya at mas lalong nadagdagan ang self-confidence ko dahil nagkaroon ako ng pagkakataon na makatrabaho ang nag-iisang superstar." Proud siya na kinatawan niya ang bansa sa nasabing international film festival. "It's such a blessing to experience attending this film festival. I was able to meet the stars and directors from different countries at paniguradong isa ito sa highlights ng aking career bilang isang aktor. The experience inspires me to do more and be the best that I can be." Samantala, napansin naman ng isang Vietnamese entertainment website na si Alden at tinawag pa nila itong "Dien vien noi tieng cua" o sa Ingles ay Philippines' Famous Actor.</t>
         </is>
       </c>
       <c r="C467" s="2" t="inlineStr">
@@ -12307,7 +12307,7 @@
       </c>
       <c r="B474" s="3" t="inlineStr">
         <is>
-          <t>IPINALIWANAG ng Palasyo na nagdesisyon si Pangulong Duterte na i-veto ang panukalang batas sa coconut levy dahil matutulad lamang daw ito sa kontrobersiyal na Road Board kung saan napunta sa katiwalian ang pondo. Ani Presidential Spokesperson at Chief Presidential Legal Counsel Salvador Panelo na sa ilalim ng panukalang Revised Coconut Industry Code ay maglalaan ng P10 bilyon ang gobyerno na hahawakan ng PCA Board. "The PCA is set up like the Road Board which is heavily criticized for allegations of corruption and misappropriation of funds. The PCA Board, like the Road Board which disburses the Motor Vehicle User's Charge, is given full authority to disburse P10-billion every year in perpetuity without a terminal date, and subject only to review by Congress after six years," sabi ni Pa-nelo. Nauna nang nagpadala ng liham si Duterte sa Senado at Kamara kaugnay sa kanyang desisyong huwag lagdaan ang isinumiteng panukala sa Palasyo. "While the President recognizes and commends the efforts of both Houses for their zealousness and selflessness in passing the measure, it is therefore with a heavy heart that he exercises his veto power pursuant to Article 6, Section 27, Paragraph 1 of the Constitution over the said bill, with the thought and confidence that the lawmakers can re-craft one that will provide more safeguards to protect the taxpayers' money and shield the levy funds from irregular and unlawful use, as well as guarantee its proper management," ayon pa sa opisyal.</t>
+          <t>IPINALIWANAG ng Palasyo na nagdesisyon si Pangulong Duterte na i-veto ang panukalang batas sa coconut levy dahil matutulad lamang daw ito sa kontrobersiyal na Road Board kung saan napunta sa katiwalian ang pondo. Ani Presidential Spokesperson at Chief Presidential Legal Counsel Salvador Panelo na sa ilalim ng panukalang Revised Coconut Industry Code ay maglalaan ng P10 bilyon ang gobyerno na hahawakan ng PCA Board. "The PCA is set up like the Road Board which is heavily criticized for allegations of corruption and misappropriation of funds. The PCA Board, like the Road Board which disburses the Motor Vehicle User's Charge, is given full authority to disburse P10-billion every year in perpetuity without a terminal date, and subject only to review ," sabi ni Pa-nelo. Nauna nang nagpadala ng liham si Duterte sa Senado at Kamara kaugnay sa kanyang desisyong huwag lagdaan ang isinumiteng panukala sa Palasyo. "While the President recognizes and commends the efforts of both Houses for their zealousness and selflessness in passing the measure, it is therefore with a heavy heart that he exercises his veto power pursuant to Article 6, Section 27, Paragraph 1 of the Constitution over the said bill, with the thought and confidence that the lawmakers can re-craft one that will provide more safeguards to protect the taxpayers' money and shield the levy funds from irregular and unlawful use, as well as guarantee its proper management," ayon pa sa opisyal.</t>
         </is>
       </c>
       <c r="C474" s="2" t="inlineStr">
@@ -12782,7 +12782,7 @@
       </c>
       <c r="B493" s="3" t="inlineStr">
         <is>
-          <t>ILANG shooting days na lang, matatapos na ang MMFF entry ng Star Cinema starring Vice Ganda, Richard Yap at Bimby Yap na The Amazing: Praybeyt Benjamin na nagpresscon na kahapon. Kung ganado sa shooting si Vice, mas ganado si Sir Chief kaya nakapag-comment ang una na ang galing-galing ni Richard sa nasabing movie.</t>
+          <t>ILANG shooting days na lang, matatapos na ang MMFF entry ng Star Cinema starring Vice Ganda, Richard Yap at Bim : Praybeyt Benjamin na nagpresscon na kahapon. Kung ganado sa shooting si Vice, mas ganado si Sir Chief kaya nakapag-comment ang una na ang galing-galing ni Richard sa nasabing movie.</t>
         </is>
       </c>
       <c r="C493" s="2" t="inlineStr">
@@ -12957,7 +12957,7 @@
       </c>
       <c r="B500" s="3" t="inlineStr">
         <is>
-          <t>Inakusahan ng dating kongresista at dating Technical education and Skills Development Authority (TESDA) chief na si Augusto Syjuco Jr. si Purisima ng pagganap sa tungkulin kahit na suspendido ito, at si Napenas dahil sa pagsunod sa utos ng heneral. Sa 15-pahinang reklamo, inakusahan ni Syjuco si Purisima ng paglabag sa Anti-Graft and Corrupt Practices Act sa pakikialam sa Oplan Exodus kahit na suspendido sa tungkulin noon pang Disyembre 2014. Sinabi ni Syjuco na mismong si Pangulong Benigno S. Aquino III ay umamin na may "lack of coordination" sa puwersa ng gobyerno at sa Moro Islamic Liberation Front (MILF) nang isagawa ang Oplan Exodus at alam din ni Purisima ang tungkol sa operasyon na hindi ipinabatid kina Interior and Local Government (DILG) Secretary Manuel Roxas at acting PNP chief Deputy Director Gen. Leonardo Espina. "As many claimed, Purisima not only knew of the operation, but actually controlled and directed the operations, despite his being currently suspended from duty," ani Syjuco. Dagdag niya, "The fatal covert operation that killed 44 members of the elite SAF had been assigned by President Benigno Aquino to suspended National Police Chief Alan Purisima, apparently without the knowledge of Interior Secretary Manuel 'Mar' Roxas. On this point alone, it may well be said that Aquino considered Purisima as still the 'de facto PNP chief' in assigning to him the sensitive mission, despite his suspended status," saad sa reklamo. Giit ni Syjuco, marami at malinaw ang mga ebidensiya na nagpapatunay na pinangasiwaan nga ni Purisima ang operasyon sa Mamasapano kahit pa suspendido ito ng Ombudsman.</t>
+          <t>Inakusahan ng dating kongresista at dating Technical education and Skills Development Authority (TESDA) chief na si Augusto Syjuco Jr. si Purisima ng pagganap sa tungkulin kahit na suspendido ito, at si Napenas dahil sa pagsunod sa utos ng heneral. Sa 15-pahinang reklamo, inakusahan ni Syjuco si Purisima ng paglabag sa Anti-Graft and Corrupt Practices Act sa pakikialam sa Oplan Exodus kahit na suspendido sa tungkulin noon pang Disyembre 2014. Sinabi ni Syjuco na mismong si Pangulong Benigno S. Aquino III ay umamin na may "lack of coordination" sa puwersa ng gobyerno at sa Moro Islamic Liberation Front (MILF) nang isagawa ang Oplan Exodus at alam din ni Purisima ang tungkol sa operasyon na hindi ipinabatid kina Interior and Local Government (DILG) Secretary Manuel Roxas at acting PNP chief Deputy Director Gen. Leonardo Espina. "As many claimed, Purisima not only knew of the operation, but actually controlled and directed the operations, despite his being currently suspended from duty," ani Syjuco. Dagdag niya, "The fatal covert operation that killed 44 members of the elite SAF had been assigned ional Police Chief Alan Purisima, apparently without the knowledge of Interior Secretary Manuel 'Mar' Roxas. On this point alone, it may well be said that Aquino considered Purisima as still the 'de facto PNP chief' in assigning to him the sensitive mission, despite his suspended status," saad sa reklamo. Giit ni Syjuco, marami at malinaw ang mga ebidensiya na nagpapatunay na pinangasiwaan nga ni Purisima ang operasyon sa Mamasapano kahit pa suspendido ito ng Ombudsman.</t>
         </is>
       </c>
       <c r="C500" s="2" t="inlineStr">
@@ -13332,7 +13332,7 @@
       </c>
       <c r="B515" s="3" t="inlineStr">
         <is>
-          <t>Kaya naman masaya siya, at aminadong feeling leading man na, nang dumating siya sa second presscon niya for that day nitong Martes. Una ang presscon nila ng leading lady niyang si Valeen Montenegro para sa movie nilang The Write Moment, na ipalalabas na, produced by IdeaFirst Company at Viva Entertainment. Ipinalabas na last year ang nasabing pelikula sa Quezon City Film Festival. Kuwento ni Jerald, sa movie ay gagampanan niya ang karakter ni Dave, isang professional wedding videographer na sideline ang pagiging movie scriptwriter. Girlfriend niya si Valeen, as Joyce, na bigla na lamang siyang hiniwalayan nang walang dahilan. Hindi niya matanggap iyon, kaya naman napasulat tuloy sila ng movie script para sa kanilang dalawa ni Joyce, ang kaibahan, happy ang ending ng isinulat niyang story. Sa huli, na-realize niya na kailangan lang pala niyang sundin ang sarili niyang script para magkatuluyan sila. Ang daming hugot lines sa movie na tiyak na magugustuhan ng mga manonood. Sa direksiyon ni Dominic Lim, showing na ang The Write Moment sa Wednesday, June 27, in cinemas nationwide. May premiere night sila sa Monday, June 25, sa Robinson's Galleria. "Sa palagay ko po, sa The Write Moment ay nabuksan ang doors sa akin, na puwede pala akong maging leading man," biro ni Jerald. "Kaya very thankful po ako na in-accept nila ako, na from drama sa theatre, nagpapatawa ako. At kita poi to sa live audience sa Sunday Pinasaya ng GMA-7. "May gagawin din akong three movies, ang Nakalimutan Kong Kalimutan Ka with Alex Gonzaga at Vin Abrenica; Pangarap kong Holdup with Paolo Contis; at Mina Anod with Dennis Trillo. "Sa Real, Quezon kami magsu-shoot (ni Dennis), dahil tungkol sa surfing ang story nito. Sa August po ay mapapanood na rin ako sa Rak of Aegis sa PETA, sa third year na presentation nito." Kumusta naman ang love life ni Jerald, may gusto ba talaga siya kay Valeen? "Hindi po totoo, kulitan lang naming 'yun ni Valeen sa Sunday Pinasaya. Nagkikita pa rin kami ng French girlfriend ko, like noong minsang dumating siya, kasama ang boyfriend niya," kuwento pa ni Jerald. "Dati ay pinasusunod niya ako sa France, pero hindi ko ginawa. Sayang naman 'yung career ko rito, na medyo bumobongga na ngayon. "Mas gusto kong mabigyan muna ng magandang buhay ang pamilya ko. Gusto kong mabigyan ng bahay ang nanay ko at maipasyal siya sa ibang bansa kapag nakaipon pa ako," seryoso nang sabi ni Jerald.</t>
+          <t>Kaya naman masaya siya, at aminadong feeling leading man na, nang dumating siya sa second presscon niya for that day nitong Martes. Una ang presscon nila ng leading lady niyang si Valeen Montenegro para sa movie nilang The Write Moment, na ipalalabas na, produced Ipinalabas na last year ang nasabing pelikula sa Quezon City Film Festival. Kuwento ni Jerald, sa movie ay gagampanan niya ang karakter ni Dave, isang professional wedding videographer na sideline ang pagiging movie scriptwriter. Girlfriend niya si Valeen, as Joyce, na bigla na lamang siyang hiniwalayan nang walang dahilan. Hindi niya matanggap iyon, kaya naman napasulat tuloy sila ng movie script para sa kanilang dalawa ni Joyce, ang kaibahan, happy ang ending ng isinulat niyang story. Sa huli, na-realize niya na kailangan lang pala niyang sundin ang sarili niyang script para magkatuluyan sila. Ang daming hugot lines sa movie na tiyak na magugustuhan ng mga manonood. Sa direksiyon ni Dominic Lim, showing na ang The Write Moment sa Wednesday, June 27, in cinemas nationwide. May premiere night sila sa Monday, June 25, sa Robinson's Galleria. "Sa palagay ko po, sa The Write Moment ay nabuksan ang doors sa akin, na puwede pala akong maging leading man," biro ni Jerald. "Kaya very thankful po ako na in-accept nila ako, na from drama sa theatre, nagpapatawa ako. At kita poi to sa live audience sa Sunday Pinasaya ng GMA-7. "May gagawin din akong three movies, ang Nakalimutan Kong Kalimutan Ka with Alex Gonzaga at Vin Abrenica; Pangarap kong Holdup with Paolo Contis; at Mina Anod with Dennis Trillo. "Sa Real, Quezon kami magsu-shoot (ni Dennis), dahil tungkol sa surfing ang story nito. Sa August po ay mapapanood na rin ako sa Rak of Aegis sa PETA, sa third year na presentation nito." Kumusta naman ang love life ni Jerald, may gusto ba talaga siya kay Valeen? "Hindi po totoo, kulitan lang naming 'yun ni Valeen sa Sunday Pinasaya. Nagkikita pa rin kami ng French girlfriend ko, like noong minsang dumating siya, kasama ang boyfriend niya," kuwento pa ni Jerald. "Dati ay pinasusunod niya ako sa France, pero hindi ko ginawa. Sayang naman 'yung career ko rito, na medyo bumobongga na ngayon. "Mas gusto kong mabigyan muna ng magandang buhay ang pamilya ko. Gusto kong mabigyan ng bahay ang nanay ko at maipasyal siya sa ibang bansa kapag nakaipon pa ako," seryoso nang sabi ni Jerald.</t>
         </is>
       </c>
       <c r="C515" s="2" t="inlineStr">
@@ -13657,7 +13657,7 @@
       </c>
       <c r="B528" s="3" t="inlineStr">
         <is>
-          <t>"Ang bongga rito, ni-restore sa high definition ang mga mapapanood na pelikula, ang Anak na dinirek ni Rory Quintos; Kapag Langit Ang Humatol directed by Laurice Guillen at Bata, Bata, Paano Ka Ginawa? ni Direk Chito Rono,"sabi ni Jojo.</t>
+          <t>"Ang bongga rito, ni-restore sa high definition ang mga mapapanood na pelikula, ang Anak na dinirek ni Rory Quintos; Kapag Langit Ang Humatol directed , Bata, Paano Ka Ginawa? ni Direk Chito Rono,"sabi ni Jojo.</t>
         </is>
       </c>
       <c r="C528" s="2" t="inlineStr">
@@ -14407,7 +14407,7 @@
       </c>
       <c r="B558" s="3" t="inlineStr">
         <is>
-          <t>ISINAPUBLIKO ng Quezon City Police District (QCPD) ang composite sketch ng isa sa mga itinuturong pumatay kay Barangay Bagong Silangan chair Crisell Beltran. Sinabi ni QCPD Director Chief Supt. Joselito Esquivel Jr. ginawa ang sketch matapos makalap ang testimonya mula sa isang testigo na nakakita ng pananambang. Idinagdag ni Esquivel na umabot na sa 11 testigo ang nakuhaan ng pahayag. Ani Esquivel, nakita ng isa sa mga testigo ang mukha ng gunman nang tanggalin nito ang kanyang helmet para maglagay ng bala. Idinagdag ni Esquivel na anim na suspek ang tinitingnang bilang ng mga sangkot sa krimen matapos namang tambangan ang sinasakyan ni Beltran at kanyang driver na si Melchor Salita habang  binabagtas ang kahabaan ng J.P. Rizal st. sa Barangay Bagong Silangan noong Miyerkules. Sinabi pa ni Esquivel na apat ang tinitingnang anggulo sa pagpatay kabilang ang pulitika, negosyo, ang kaugnayan ni Beltran sa mga illegal settlers, at love angle. "[Tinitingnan] natin dito [ang] apat na direksyon ng imbestigasyon. Meron na rin tayong tinitingnan na persons of interest (We are looking at four directions of the investigation. We also have persons of interest)," sabi ni Esquivel. Itinaas na sa P5 milyon ang pabuya para sa makakapagbigay ng impormasyon para mahuli ang mga suspek.</t>
+          <t>ISINAPUBLIKO ng Quezon City Police District (QCPD) ang composite sketch ng isa sa mga itinuturong pumatay kay Barangay Bagong Silangan chair Crisell Beltran. Sinabi ni QCPD Director Chief Supt. Joselito Esquivel Jr. ginawa ang sketch matapos makalap ang testimonya mula sa isang testigo na nakakita ng pananambang. Idinagdag ni Esquivel na umabot na sa 11 testigo ang nakuhaan ng pahayag. Ani Esquivel, nakita ng isa sa mga testigo ang mukha ng gunman nang tanggalin nito ang kanyang helmet para maglagay ng bala. Idinagdag ni Esquivel na anim na suspek ang tinitingnang bilang ng mga sangkot sa krimen matapos namang tambangan ang sinasakyan ni Beltran at kanyang driver na si Melchor Salita habang binabagtas ang kahabaan ng J.P. Rizal st. sa Barangay Bagong Silangan noong Miyerkules. Sinabi pa ni Esquivel na apat ang tinitingnang anggulo sa pagpatay kabilang ang pulitika, negosyo, ang kaugnayan ni Beltran sa mga illegal settlers, at love angle. "[Tinitingnan] natin dito [ang] apat na direksyon ng imbestigasyon. Meron na rin tayong tinitingnan na persons of interest (We are looking at four directions of the investigation. We also have persons of interest)," sabi ni Esquivel. Itinaas na sa P5 milyon ang pabuya para sa makakapagbigay ng impormasyon para mahuli ang mga suspek.</t>
         </is>
       </c>
       <c r="C558" s="2" t="inlineStr">
@@ -14857,7 +14857,7 @@
       </c>
       <c r="B576" s="3" t="inlineStr">
         <is>
-          <t>Sa unang pagkakataon, masasaksihan ang love team nina Jake Vargas at Bea Binene sa kakaibang konsepto ng pelikula na malayung-malayo sa mga pa-sweet at pa-cute na mga movies at TV shows na kanilang pinagsamahan. Kumbaga, isa itong malaking hakbang tungo sa mas malaking challenges at pagle-level up sa career para sa tinanghal na Yahoo Celebrity Couple of 2014 ang hatid ng movie. Kasama nina Jake at Bea sina Igi Boy Flores at Sarah Lahbati na napasabak din sa non-stop adventures na ikagigitla at ikasisindak ng manonood! Ayon kay Direk Richard Sommes, saktung-sakto si Jake sa kanyang role bilang isang pasaway na teenager na walang pakialam sa kanyang responsibilidad. Perfect and beautiful naman ang deskripsyon kina Bea at Sarah habang si Igi Boy naman ay umakma sa role niyang nerd na natural na natural ang husay sa pagbibitiw ng punchlines. "They are also fresh and exciting faces sa screen. This is a coming of age movie na matagal ko nang gustong gawin in the tradition of foreign films like Stand By Me. Gusto kong ihatid na as teenager or young adult, they each have responsibilities sa mundo nilang ginagalawan," katwiran ni Direk Richard</t>
+          <t>Sa unang pagkakataon, masasaksihan ang love team nina Jake Vargas at Bea Binene sa kakaibang konsepto ng pelikula na malayung-malayo sa mga pa-sweet at pa-cute na mga movies at TV shows na kanilang pinagsamahan. Kumbaga, isa itong malaking hakbang tungo sa mas malaking challenges at pagle-level up sa career para sa tinanghal na Yahoo Celebrity Couple of 2014 ang hatid ng movie. Kasama nina Jake at Bea sina Igi Boy Flores at Sarah Lahbati na napasabak din sa non-stop adventures na ikagigitla at ikasisindak ng manonood! Ayon kay Direk Richard Sommes, saktung-sakto si Jake sa kanyang role bilang isang pasaway na teenager na walang pakialam sa kanyang responsibilidad. Perfect and beautiful naman ang deskripsyon kina Bea at Sarah habang si Igi Boy naman ay umakma sa role niyang nerd na natural na natural ang husay sa pagbibitiw ng punchlines. "They are also fresh and exciting faces sa screen. This is a coming of age movie na matagal ko nang gustong gawin in the tradition of foreign films like Stand oung adult, they each have responsibilities sa mundo nilang ginagalawan," katwiran ni Direk Richard</t>
         </is>
       </c>
       <c r="C576" s="2" t="inlineStr">
@@ -15582,7 +15582,7 @@
       </c>
       <c r="B605" s="3" t="inlineStr">
         <is>
-          <t>KINUMPIRMA ng Palasyo na tumulak pa-Hong Kong si Pangulong Duterte kasama ang kanyang long-time partner na si Honeylet Avancena at bunsong anak na si Kitty para magbakasyon. Sinabi ni Presidential Spokesperson and Chief Presidential Legal Counsel Salvador Panelo na regalo ito ni Duterte kay Honeylet na nagdiriwang ng kanyang kaarawan.  "Yup. He is in Hong Kong with Honeylet. It's the latter's birthday today," sabi ni Panelo.  Sinabi naman ni dating Special Assistant to the President Christopher "Bong" Go na si Kitty ang humiling sa kanilang bakasyon sa Hong Kong. "It was actually Kitty who requested her father for the trip, as a gift. Nagawa na ito nila noon kahit nung Mayor pa ng Davao City si PRRD. The weekend getaway is for rest and recreation," sabi ni Go. idinagdag ni Go na itinalaga ni Duterte si  Executive Secretary Salvador Medialdea bilang officer in charge. Umalis ang First Family kahapon at nakatakdang bumalik bukas, ayon pa kay Go.</t>
+          <t>KINUMPIRMA ng Palasyo na tumulak pa-Hong Kong si Pangulong Duterte kasama ang kanyang long-time partner na si Honeylet Avancena at bunsong anak na si Kitty para magbakasyon. Sinabi ni Presidential Spokesperson and Chief Presidential Legal Counsel Salvador Panelo na regalo ito ni Duterte kay Honeylet na nagdiriwang ng kanyang kaarawan. "Yup. He is in Hong Kong with Honeylet. It's the latter's birthday today," sabi ni Panelo. Sinabi naman ni dating Special Assistant to the President Christopher "Bong" Go na si Kitty ang humiling sa kanilang bakasyon sa Hong Kong. "It was actually Kitty who requested her father for the trip, as a gift. Nagawa na ito nila noon kahit nung Mayor pa ng Davao City si PRRD. The weekend getaway is for rest and recreation," sabi ni Go. idinagdag ni Go na itinalaga ni Duterte si Executive Secretary Salvador Medialdea bilang officer in charge. Umalis ang First Family kahapon at nakatakdang bumalik bukas, ayon pa kay Go.</t>
         </is>
       </c>
       <c r="C605" s="2" t="inlineStr">
@@ -16857,7 +16857,7 @@
       </c>
       <c r="B656" s="3" t="inlineStr">
         <is>
-          <t>Sa unang pagkakataon, napanood ng publiko ang digitally restored at remastered na mga kopya ng Anak directed by Rory Quintos, Kapag Langit ang Humatol directed by Laurice Guillen at Bata, Bata, Paano ka Ginawa ni Chito Rono. Mabusising inayos, pinalinaw at pinaganda ng ABS-CBN Film Archives at Central Digita Labs ang naturang mga pelikula. Dumating ang ilang ABS-CBN executives at director na kinabibilangan nina Ms. Malou Santos, Chit Guerrero, Olive Lamasan, Rory Quintos, Laurice Guillen at Chito Rono sa UP Film Center para panoorin ang Bata, Bata.... Dumating din sina Cherrie Pie Picache at Albert Martinez, na kasama sa cast nito. In full force din na dumating sa event ang Vilmanians at press people. Sa totoo lang, aakalain mong bago ang kopya ng restored films. Kung hindi nga lang naroroon sina Carlo Aquino at Serena Dalrymple na mga totoy at nene pa ang itsura sa movie, aakalain mong bagong pelikula ang Bata... Bata.... Salamat sa modernong teknolohiya. Sabi sa speech ni Leo Katigbak, ang ABS-CBN Film Archives head, anim nang classic film ni Ate Vi ang na-restore nila at baka nga lumobo pa ito sa maraming kopya dahil sa magandang pagtanggap ng publiko. Sa talumpati naman ni Ate Vi, aniyang pabiro, "Anim pa lang? Bakit hindi 15?" At idinagdag na, "Modesty aside, marami tayong classic films na nagawa na kailangan munang i-restore dahil sa kalumaan." "Gusto naming i-restore ang mga natatanging pelikula ni Vilma mula sa iba't ibang direktor," kuwento pa ni Mr. Katigbak. All in all, nakapag-restore na ang ABS-CBN Film Archives ng 72 pelikula since 2011 at ang ilan sa mga ito ay pinalad na maipalabas sa international filmfest at sa katunayan ay may red-carpet pang premiere na naganap at naiere sa free-to-air/cable television. Napapanood din ang mga ito sa pay-per-view at video-on-demand, nabibili sa DVD at nada-download din sa iTunes. Sa tanong kay Ate Vi kung ano pa ang nagawa niyang pelikula na gusto niyang panoorin, ang excited niyang sagot, "T-Bird at Ako."</t>
+          <t>Sa unang pagkakataon, napanood ng publiko ang digitally restored at remastered na mga kopya ng Anak directed , Kapag Langit ang Humatol directed , Bata, Paano ka Ginawa ni Chito Rono. Mabusising inayos, pinalinaw at pinaganda ng ABS-CBN Film Archives at Central Digita Labs ang naturang mga pelikula. Dumating ang ilang ABS-CBN executives at director na kinabibilangan nina Ms. Malou Santos, Chit Guerrero, Olive Lamasan, Rory Quintos, Laurice Guillen at Chito Rono sa UP Film Center para panoorin ang Bata, Bata.... Dumating din sina Cherrie Pie Picache at Albert Martinez, na kasama sa cast nito. In full force din na dumating sa event ang Vilmanians at press people. Sa totoo lang, aakalain mong bago ang kopya ng restored films. Kung hindi nga lang naroroon sina Carlo Aquino at Serena Dalrymple na mga totoy at nene pa ang itsura sa movie, aakalain mong bagong pelikula ang Bata... Bata.... Salamat sa modernong teknolohiya. Sabi sa speech ni Leo Katigbak, ang ABS-CBN Film Archives head, anim nang classic film ni Ate Vi ang na-restore nila at baka nga lumobo pa ito sa maraming kopya dahil sa magandang pagtanggap ng publiko. Sa talumpati naman ni Ate Vi, aniyang pabiro, "Anim pa lang? Bakit hindi 15?" At idinagdag na, "Modesty aside, marami tayong classic films na nagawa na kailangan munang i-restore dahil sa kalumaan." "Gusto naming i-restore ang mga natatanging pelikula ni Vilma mula sa iba't ibang direktor," kuwento pa ni Mr. Katigbak. All in all, nakapag-restore na ang ABS-CBN Film Archives ng 72 pelikula since 2011 at ang ilan sa mga ito ay pinalad na maipalabas sa international filmfest at sa katunayan ay may red-carpet pang premiere na naganap at naiere sa free-to-air/cable television. Napapanood din ang mga ito sa pay-per-view at video-on-demand, nabibili sa DVD at nada-download din sa iTunes. Sa tanong kay Ate Vi kung ano pa ang nagawa niyang pelikula na gusto niyang panoorin, ang excited niyang sagot, "T-Bird at Ako."</t>
         </is>
       </c>
       <c r="C656" s="2" t="inlineStr">
@@ -16882,7 +16882,7 @@
       </c>
       <c r="B657" s="3" t="inlineStr">
         <is>
-          <t>"Reports that I was sneaked out by PNP personnel from the Custodial Center are absolutely false," pahayag ni Revilla. Una nang napaulat na umalis si Revilla mula sa detention compound noong Valentine's Day, Pebrero 14, upang bisitahin si Enrile, na may kaarawan ng araw na iyon. Sina Enrile, Revilla at Sen. Jose "Jinggoy" Estrada ay pawang nakakulong sa PNP headquarters dahil sa pagkakasangkot nila sa P10-bilyon pork barrel fund scam. Dakong 3:00 ng hapon ng nasabing araw, ayon kay Revilla, ay isinugod siya sa PNP General Hospital makaraan niyang magpawis nang malamig, makaramdam ng paninigas at pananakit ng leeg, batok at likod, at matinding migraine attack. "It appeared that I had a spike in my blood pressure," aniya. "I was taken to the hospital by Custodial Center Guards after a written request was made to Col. Fabro, the Director of the Custodial Center. I was accompanied by my two children, Bryan and Vice Gov. Jolo," dagdag ng senador. Sinabi ni Revilla na maging ang PNP ay nilinaw na ang isyu. "I stayed in the hospital for less than 30 minutes and I was immediately taken back to my detention cell to rest, after my blood pressure was taken and injected with medication," sabi niya.</t>
+          <t>"Reports that I was sneaked out re absolutely false," pahayag ni Revilla. Una nang napaulat na umalis si Revilla mula sa detention compound noong Valentine's Day, Pebrero 14, upang bisitahin si Enrile, na may kaarawan ng araw na iyon. Sina Enrile, Revilla at Sen. Jose "Jinggoy" Estrada ay pawang nakakulong sa PNP headquarters dahil sa pagkakasangkot nila sa P10-bilyon pork barrel fund scam. Dakong 3:00 ng hapon ng nasabing araw, ayon kay Revilla, ay isinugod siya sa PNP General Hospital makaraan niyang magpawis nang malamig, makaramdam ng paninigas at pananakit ng leeg, batok at likod, at matinding migraine attack. "It appeared that I had a spike in my blood pressure," aniya. "I was taken to the hospital equest was made to Col. Fabro, the Director of the Custodial Center. I was accompanied by my two children, Bryan and Vice Gov. Jolo," dagdag ng senador. Sinabi ni Revilla na maging ang PNP ay nilinaw na ang isyu. "I stayed in the hospital for less than 30 minutes and I was immediately taken back to my detention cell to rest, after my blood pressure was taken and injected with medication," sabi niya.</t>
         </is>
       </c>
       <c r="C657" s="2" t="inlineStr">
@@ -16907,7 +16907,7 @@
       </c>
       <c r="B658" s="3" t="inlineStr">
         <is>
-          <t>NAIS itama ng Bandera ang pagkakamali sa isang istorya nito na  naipost sa website noong Pebrero 4. Nagpapasalamat ang Bandera kay Sheila Mateo, kamag-anak ng pinaslang na si Boyet San Buenaventura, sa pagtawag sa atensyon sa Bandera ukol sa pagkakamali nito. Si San Buenaventura ang may-ari ng tindahan na pinaslang umano ng bumibili na si Jessie Mark Batugon; at hindi gaya nang napaunang ulat hindi lang Bandera kundi sa iba pang mga news website. (Read more) http://https://bandera.inquirer.net/208320/lalaking-bumili-ng-noodles-patay-matapos-barilin-ng-may-ari-ng-tindahan-sa-quezon Narito ang itinamang istorya: PATAY ang isang 37-anyos na lalaki matapos barilin sa kanyang tindahan sa Gumaca, Quezon bago maghatinggabi noong Linggo, Pebrero 3, ayon sa pulisya. Kinilala ni Senior Supt. Osmundo de Guzman, Quezon police director, ang nasawi na Boyet San Buenaventura. Isang police manhunt naman ang inilunsad laban sa suspek na si Jessie Mark Batugon, 19, sa Barangay Progreso. Sa kuwento ng kamag-anak ng biktima na si Sheila Mateo, pumunta si Batugon sa tindahan upang bumili ng noodles. Ang nagbabantay sa tindahan ay ang misis ng nasawi na si Cristina. Nakita umano ng suspek ang biktima na nagtungo sa likuran ng tindahan at doon ay umiihi; pinuntahan ito ng suspek at doon binaril ang biktima sa likod gamit ang .22 kalibreng baril. Binawian ng buhay ang biktima habang dinadala sa San Diego Hospital. Narekober ng mga pulis ang baril, bagamat nakatakas ang suspek. Nanawagan ng hustisya ang mga kamag-anak ng biktima</t>
+          <t>NAIS itama ng Bandera ang pagkakamali sa isang istorya nito na naipost sa website noong Pebrero 4. Nagpapasalamat ang Bandera kay Sheila Mateo, kamag-anak ng pinaslang na si Boyet San Buenaventura, sa pagtawag sa atensyon sa Bandera ukol sa pagkakamali nito. Si San Buenaventura ang may-ari ng tindahan na pinaslang umano ng bumibili na si Jessie Mark Batugon; at hindi gaya nang napaunang ulat hindi lang Bandera kundi sa iba pang mga news website. (Read more) Narito ang itinamang istorya: PATAY ang isang 37-anyos na lalaki matapos barilin sa kanyang tindahan sa Gumaca, Quezon bago maghatinggabi noong Linggo, Pebrero 3, ayon sa pulisya. Kinilala ni Senior Supt. Osmundo de Guzman, Quezon police director, ang nasawi na Boyet San Buenaventura. Isang police manhunt naman ang inilunsad laban sa suspek na si Jessie Mark Batugon, 19, sa Barangay Progreso. Sa kuwento ng kamag-anak ng biktima na si Sheila Mateo, pumunta si Batugon sa tindahan upang bumili ng noodles. Ang nagbabantay sa tindahan ay ang misis ng nasawi na si Cristina. Nakita umano ng suspek ang biktima na nagtungo sa likuran ng tindahan at doon ay umiihi; pinuntahan ito ng suspek at doon binaril ang biktima sa likod gamit ang .22 kalibreng baril. Binawian ng buhay ang biktima habang dinadala sa San Diego Hospital. Narekober ng mga pulis ang baril, bagamat nakatakas ang suspek. Nanawagan ng hustisya ang mga kamag-anak ng biktima</t>
         </is>
       </c>
       <c r="C658" s="2" t="inlineStr">
@@ -17257,7 +17257,7 @@
       </c>
       <c r="B672" s="3" t="inlineStr">
         <is>
-          <t>NAIS ng prosekusyon na pabayaran na kay dating Sen. Ramon Bong Revilla Jr., at mga kapwa akusado nito ang P124.3 milyong pondo ng gobyerno na nawala dahil sa pork barrel fund scam. Sinabi ng prosekusyon na bagamat pinawalang-sala si Revilla sa kasong kriminal nakasaad sa naturang desisyon na "accused are held solidarily and jointly liable to return to the National Treasury the amount of One-Hundred Twenty-four million, Five hundred Thousand pesos". Ang mga kapwa akusado ni Revilla na sina Janet Lim Napoles at Richard Cambe, dating aide ng senador, ay hinatulan ng habambuhay na pagkakakulong. "As regards Revilla, while he was acquitted, the same was based merely on reasonable doubt and not due to the absolute failure of the prosecution to prove his guilt. This is why the judgment did not declare him to without civil liability," saad ng prosekusyon sa inihain nitong mosyon. Ginamit din ng prosekusyon sa kanilang argumento ang Article 100 ng Revised Penal Code na hindi nagsasabi na ang maaari lamang civilly liable ay ang mga criminally liable. "Thus, a person acquitted may still be civilly liable if there is basis to hold him/her so.  Courts can acquit an accused on reasonable doubt but still order payment of civil damages in the same case. That is what the majority did in the present case."</t>
+          <t>NAIS ng prosekusyon na pabayaran na kay dating Sen. Ramon Bong Revilla Jr., at mga kapwa akusado nito ang P124.3 milyong pondo ng gobyerno na nawala dahil sa pork barrel fund scam. Sinabi ng prosekusyon na bagamat pinawalang-sala si Revilla sa kasong kriminal nakasaad sa naturang desisyon na "accused are held solidarily and jointly liable to return to the National Treasury the amount of One-Hundred Twenty-four million, Five hundred Thousand pesos". Ang mga kapwa akusado ni Revilla na sina Janet Lim Napoles at Richard Cambe, dating aide ng senador, ay hinatulan ng habambuhay na pagkakakulong. "As regards Revilla, while he was acquitted, the same was based merely on reasonable doubt and not due to the absolute failure of the prosecution to prove his guilt. This is why the judgment did not declare him to without civil liability," saad ng prosekusyon sa inihain nitong mosyon. Ginamit din ng prosekusyon sa kanilang argumento ang Article 100 ng Revised Penal Code na hindi nagsasabi na ang maaari lamang civilly liable ay ang mga criminally liable. "Thus, a person acquitted may still be civilly liable if there is basis to hold him/her so. Courts can acquit an accused on reasonable doubt but still order payment of civil damages in the same case. That is what the majority did in the present case."</t>
         </is>
       </c>
       <c r="C672" s="2" t="inlineStr">
@@ -17782,7 +17782,7 @@
       </c>
       <c r="B693" s="3" t="inlineStr">
         <is>
-          <t>KAHON-kahong pekeng panty liner na nagkakahaga ng mahigit P60,000 ang nakumpiska ng mga tauhan ng National Bureau of Investigation-Intellectual Property Rights Division (NBI-IPRD) sa raid sa Antipolo City, Rizal. Ayon kay Isaac Carpeso, team leader ng NBI-IPRD na nagsagawa ng operasyon, alas-2 ng hapon kamakalawa nang salakayin ang Misumi Direct Sales sa Unit 5, Okinari Building, Circumferential Road, Antipolo, sa bisa ng search warrant na inisyu ng Manila Regional Trial Court branch 46. Ang naturang establisimento, na pag-aari ni Donnah Mae Miranda, ay nakuhanan ng mahigit limang kahon ng pekeng Shuya panty liner. Ani Carpeso, isinagawa ang operasyon matapos silang makatanggap ng reklamo mula sa totoong gumagawa ng Shuya panty liner ukol sa pagkalat ng mga peke nilang produkto. Matapos ang ilang test buy, agad  na nagkasa ng operasyon ang mga operatiba na nagresulta sa pagkakumpiska ng mga nasabing pekeng produkto. Wala naman ang may-ari na si MIranda nang isagawa ang raid. Nahaharap si Miranda sa kasong paglabag sa trademark infringement o paglabag sa Republic Act 8293.</t>
+          <t>KAHON-kahong pekeng panty liner na nagkakahaga ng mahigit P60,000 ang nakumpiska ng mga tauhan ng National Bureau of Investigation-Intellectual Property Rights Division (NBI-IPRD) sa raid sa Antipolo City, Rizal. Ayon kay Isaac Carpeso, team leader ng NBI-IPRD na nagsagawa ng operasyon, alas-2 ng hapon kamakalawa nang salakayin ang Misumi Direct Sales sa Unit 5, Okinari Building, Circumferential Road, Antipolo, sa bisa ng search warrant na inisyu ng Manila Regional Trial Court branch 46. Ang naturang establisimento, na pag-aari ni Donnah Mae Miranda, ay nakuhanan ng mahigit limang kahon ng pekeng Shuya panty liner. Ani Carpeso, isinagawa ang operasyon matapos silang makatanggap ng reklamo mula sa totoong gumagawa ng Shuya panty liner ukol sa pagkalat ng mga peke nilang produkto. Matapos ang ilang test buy, agad na nagkasa ng operasyon ang mga operatiba na nagresulta sa pagkakumpiska ng mga nasabing pekeng produkto. Wala naman ang may-ari na si MIranda nang isagawa ang raid. Nahaharap si Miranda sa kasong paglabag sa trademark infringement o paglabag sa Republic Act 8293.</t>
         </is>
       </c>
       <c r="C693" s="2" t="inlineStr">
@@ -17882,7 +17882,7 @@
       </c>
       <c r="B697" s="3" t="inlineStr">
         <is>
-          <t>Gaganapin ang libreng medical mission sa Pebrero 23 hanggang Marso 3, 2015 para sa mga siyam na buwan hanggang pitong taong gulang. Maaaring tumawag sa 0918-9219463, 0906-8883926, at 0922-8490174. Para sa screening requirements ng mga pasyente, maaaring mag-email sa rcsta.rosacentro@yahoo.com o personal na magsadya sa Doray's Paanakan sa No. 784 F. Gomez Street, Barangay Ibaba, Sta. Rosa, Laguna.</t>
+          <t>Gaganapin ang libreng medical mission sa Pebrero 23 hanggang Marso 3, 2015 para sa mga siyam na buwan hanggang pitong taong gulang. Maaaring tumawag sa 0918-9219463, 0906-8883926, at 0922-8490174. Para sa screening requirements ng mga pasyente, maaaring mag-email sa o personal na magsadya sa Doray's Paanakan sa No. 784 F. Gomez Street, Barangay Ibaba, Sta. Rosa, Laguna.</t>
         </is>
       </c>
       <c r="C697" s="2" t="inlineStr">
@@ -17907,7 +17907,7 @@
       </c>
       <c r="B698" s="3" t="inlineStr">
         <is>
-          <t>Sa pang-MMFF na handog ni Bossing Vic, kasama ang mga kasosyo niyang OctoArts,APTFilms at sarili niyang M-ZetFilms, kasama niya sa tatlong episodes ng My Big Bossing si Ryzza Mae na pumapel bilang "Sirena," with Marian Rivera in "Taktak" at "Prinsesa" willi Nikki Gil. Buong-buo ang loob ni Bossing Vic na ka-tandem si Ryzza Mae sa halip na mga leading lady niyang pawang ubod ng gandang sina Marian, Nikki Gil, at Pauleen Luna. Hindi magiging buo ang pelikula o ano mang project niya ngayon kung wala si Ryzza Mae, or vice versa. "Ang wish ko this Christmas ay makasama lagi si Bossing Vic sa susunod na MMFF," ani Ryzza. Nakalimutan niyang dagdag ang "forever and ever." "Marami na po akong toys, sapatos, damit, gadgets, kaya iba naman ang wish ko. Ang makasama niyang lagi. Pati kasi bahay, lupa at Fortuner (sasakyan) ay mayroon na rin po ako. May teacher pa ako from international school na pumupunta sa bahay ko once a week. Kaya, puwede ko nang labanan si Alonzo (Muhlach) sa inglesan," patuloy niya. Noon daw kasing gawin nila ni Bimby Aquino Yap ang My Little Bossings, nag-nosebleed siya. "Ngayon, si Alonzo na ang sumusuko sa akin. Pikon na pikon 'yan kapag tinutukso ko na crush niya ako. Four years old lang kasi si Alonzo, malikot pa. Nahihilo ako sa kaiikotniya. Parang trumpo," patuloy ni Aling Maliit. Kung si Aiza ang lucky charmni Vic noong 1990s, walang dudang si Ryzza naman ang pampasuwerte niya ngayon. Naalaala ko rin si Aiza noong bata pa ito. Ayaw sa mga lamang pambabae, at "baril-barilan ang gusto ko at kotse-kotsehan" ang lagi niyang sagot kapag natatanong kung ano ang gusto niyang regalo 'pag Pasko. Iyon, noon pa man ay hinulaan na ni Bossing Vic na magiging karibal pa niya si Aiza sa mga chicks niya. Kung nasaan si Bossing Vic noon, naroon din si Aiza. Kahit noong panahong humina ang career ni Aiza dahil nagdadalaga/ nagbibinata na ay suportado pa rin siya ni Bossing Vic. Walang project sa pelikula at TV na wala si Aiza. Nariyang anak, ampon, nakababatang kapatid o ano pa man, basta nariyan siya anuman ang project ni Bossing Vic. Nitong ikasal si Aiza sa kapwa babae niyang beauty queen na si Liza Dino, nariyan pa rin si Bossing Vic.</t>
+          <t>Sa pang-MMFF na handog ni Bossing Vic, kasama ang mga kasosyo niyang OctoArts,APTFilms at sarili niyang M-ZetFilms, kasama niya sa tatlong episodes ng My Big Bossing si Ryzza Mae na pumapel bilang "Sirena," with Marian Rivera in "Taktak" at "Prinsesa" willi Nikki Gil. Buong-buo ang loob ni Bossing Vic na ka-tandem si Ryzza Mae sa halip na mga leading lady niyang pawang ubod ng gandang sina Marian, Nikki Gil, at Pauleen Luna. Hindi magiging buo ang pelikula o ano mang project niya ngayon kung wala si Ryzza Mae, or vice versa. "Ang wish ko this Christmas ay makasama lagi si Bossing Vic sa susunod na MMFF," ani Ryzza. Nakalimutan niyang dagdag ang "forever and ever." "Marami na po akong toys, sapatos, damit, gadgets, kaya iba naman ang wish ko. Ang makasama niyang lagi. Pati kasi bahay, lupa at Fortuner (sasakyan) ay mayroon na rin po ako. May teacher pa ako from international school na pumupunta sa bahay ko once a week. Kaya, puwede ko nang labanan si Alonzo (Muhlach) sa inglesan," patuloy niya. Noon daw kasing gawin nila ni Bim , nag-nosebleed siya. "Ngayon, si Alonzo na ang sumusuko sa akin. Pikon na pikon 'yan kapag tinutukso ko na crush niya ako. Four years old lang kasi si Alonzo, malikot pa. Nahihilo ako sa kaiikotniya. Parang trumpo," patuloy ni Aling Maliit. Kung si Aiza ang lucky charmni Vic noong 1990s, walang dudang si Ryzza naman ang pampasuwerte niya ngayon. Naalaala ko rin si Aiza noong bata pa ito. Ayaw sa mga lamang pambabae, at "baril-barilan ang gusto ko at kotse-kotsehan" ang lagi niyang sagot kapag natatanong kung ano ang gusto niyang regalo 'pag Pasko. Iyon, noon pa man ay hinulaan na ni Bossing Vic na magiging karibal pa niya si Aiza sa mga chicks niya. Kung nasaan si Bossing Vic noon, naroon din si Aiza. Kahit noong panahong humina ang career ni Aiza dahil nagdadalaga/ nagbibinata na ay suportado pa rin siya ni Bossing Vic. Walang project sa pelikula at TV na wala si Aiza. Nariyang anak, ampon, nakababatang kapatid o ano pa man, basta nariyan siya anuman ang project ni Bossing Vic. Nitong ikasal si Aiza sa kapwa babae niyang beauty queen na si Liza Dino, nariyan pa rin si Bossing Vic.</t>
         </is>
       </c>
       <c r="C698" s="2" t="inlineStr">
@@ -19682,7 +19682,7 @@
       </c>
       <c r="B769" s="5" t="inlineStr">
         <is>
-          <t>Blocktimer si Willie, hindi station produced ang show at tila P2M every Sunday ang production cost ng gagawing programa. Tinawagan na raw ni Willie ang mga kaibigan na gustong mag-sponsor sa kanyag shows, sila rin ang sponsors ng show noong nasa ABS-CBN at TV5 pa ang show niya. Ang pagpasok ng show ni Willie ang nakita naming rason kung bakit biglang na-move sa April ang airing ng InstaDad na naka-schedule umere ng March 22. Pagkatapos ng Sunday All Stars ang dapat na time slot ng InstaDad na time slot ngayon ng show ni Willie. Kaya ang tanong, saan na ilalagay ang InstaDad ngayon? Kung titingnan, walang problema sa airing, ibalik sa 12 ng tanghali ang SAS, saka ipasok ang Instadad at isunod ang show ni Willie o puwedeng unahin ang show ni Willie bago ang comedy show ni Gabby Eigenmann.</t>
+          <t>Blocktimer si Willie, hindi station produced ang show at tila P2M every Sunday ang production cost ng gagawing programa. Tinawagan na raw ni Willie ang mga kaibigan na gustong mag-sponsor sa kanyag shows, sila rin ang sponsors ng show noong nasa ABS-CBN at TV5 pa ang show niya. Ang pagpasok ng show ni Willie ang nakita naming rason kung bakit biglang na-move sa April ang airing ng InstaDad na naka-schedule umere ng March 22. Pagkatapos ng Sunday All Stars ang dapat na time slot ng InstaDad na time slot ngayon ng show ni Willie. Kaya ang tanong, saan na ilalagay ang InstaDad ngayon? Kung titingnan, walang problema sa airing, ibalik sa 12 ng tanghali ang SAS, saka ipasok ang Instadad at isunod ang show ni Willie o puwedeng unahin ang show ni Willie bago ang comedy show ni Gab</t>
         </is>
       </c>
       <c r="C769" s="4" t="inlineStr">
@@ -19807,7 +19807,7 @@
       </c>
       <c r="B774" s="5" t="inlineStr">
         <is>
-          <t>KAKAIBANG Lady Gaga, na talaga namang ikinagulat ng lahat, ang napanood sa 87th Academy Awards noong Linggo, Pebrero 22, nang awitin niya ang The Sound of Music medley sa Dolby Theatre sa Los Angeles. Inawit ng singer ang ilang medley song kabilang na ang The Hills Are Alive, Edelweiss at Climb Ev'ry Mountain. Ayon sa ulat ng US Weekly, ang My Favorite Things ay isa rin sa presentasyon ni Gaga -- ito ang una niyang pagtatanghal simula nang isiwalat niya noong Valentine's Day ang planong pagpapakasal sa aktor na si Taylor Kinney.</t>
+          <t>KAKAIBANG Lady Gaga, na talaga namang ikinagulat ng lahat, ang napanood sa 87th Academy Awards noong Linggo, Pebrero 22, nang awitin niya ang The Sound of Music medley sa Dol ang ilang medley song kabilang na ang The Hills Are Alive, Edelweiss at Climb Ev'ry Mountain. Ayon sa ulat ng US Weekly, ang My Favorite Things ay isa rin sa presentasyon ni Gaga -- ito ang una niyang pagtatanghal simula nang isiwalat niya noong Valentine's Day ang planong pagpapakasal sa aktor na si Taylor Kinney.</t>
         </is>
       </c>
       <c r="C774" s="4" t="inlineStr">
@@ -19957,7 +19957,7 @@
       </c>
       <c r="B780" s="5" t="inlineStr">
         <is>
-          <t>Ayon kay Inigo nang makausap namin siya sa presscon ng pelikulang Crazy Beautiful You ay natutuwa nga raw siya at isinama siya ng Star Cinema sa newest KathNiel movie. "It is an honor to be working with them. I'm very thankful that I'm part of their partnership," sey pa ni Inigo. Bukod sa kanilang tatlo ay kasama rin sa movie ng Star Cinema sina Lorna Tolentino at ama ni KC Concepcion na si Gabby Concepcion na naging kasintahan ng ama naman niyang si Piolo Pascual. Kumusta naman ang pakikipagtrabaho niya sa dalawang beteranong artista? "Well, at first, eh, I was really nervous to work with them pero nu'ng nakita ko na ang set na sobrang happy, kaya medyo nadalian akong makisama sa kanila. They were all kind and generous, so it was very easy," kuwento pa ni Inigo. Aniya pa, ibang-iba na ang ginawa niya ngayon kung ikukumpara sa naunang pelikula niya.</t>
+          <t>Ayon kay Inigo nang makausap namin siya sa presscon ng pelikulang Crazy Beautiful You ay natutuwa nga raw siya at isinama siya ng Star Cinema sa newest KathNiel movie. "It is an honor to be working with them. I'm very thankful that I'm part of their partnership," sey pa ni Inigo. Bukod sa kanilang tatlo ay kasama rin sa movie ng Star Cinema sina Lorna Tolentino at ama ni KC Concepcion na si Gab man niyang si Piolo Pascual. Kumusta naman ang pakikipagtrabaho niya sa dalawang beteranong artista? "Well, at first, eh, I was really nervous to work with them pero nu'ng nakita ko na ang set na sobrang happy, kaya medyo nadalian akong makisama sa kanila. They were all kind and generous, so it was very easy," kuwento pa ni Inigo. Aniya pa, ibang-iba na ang ginawa niya ngayon kung ikukumpara sa naunang pelikula niya.</t>
         </is>
       </c>
       <c r="C780" s="4" t="inlineStr">
@@ -20357,7 +20357,7 @@
       </c>
       <c r="B796" s="5" t="inlineStr">
         <is>
-          <t>ISANG kapitan ng barangay na tumatakbo sa pagkakongresista ang pinagbabaril at napatay ng riding-in tandem sa Quezon City ngayong araw. Dead on arrival sa FEU Hospital si Crisell 'Bheng' Beltran sanhi ng mga tama ng bala. Nasawi rin ang driver ni Beltran na si Melchor Salita na dinala sa General Malvar Hospital. Sakay si Beltran at tatlong iba pa ng puting Ford Everest (NDO 612) at binabagtas ang JP Rizal, Brgy. Bagong Silangan ng tabihan ng apat na lalaki na nakasakay ng dalawang motorsiklo alas-11:40 ng umaga. Pinagbabaril ng mga suspek ang sasakyan ng biktima. Nasugatan din sa pangyayari ang apat pang katao.  Inaalam pa ng pulisya ang motibo sa pamamaslang.</t>
+          <t>ISANG kapitan ng barangay na tumatakbo sa pagkakongresista ang pinagbabaril at napatay ng riding-in tandem sa Quezon City ngayong araw. Dead on arrival sa FEU Hospital si Crisell 'Bheng' Beltran sanhi ng mga tama ng bala. Nasawi rin ang driver ni Beltran na si Melchor Salita na dinala sa General Malvar Hospital. Sakay si Beltran at tatlong iba pa ng puting Ford Everest (NDO 612) at binabagtas ang JP Rizal, Brgy. Bagong Silangan ng tabihan ng apat na lalaki na nakasakay ng dalawang motorsiklo alas-11:40 ng umaga. Pinagbabaril ng mga suspek ang sasakyan ng biktima. Nasugatan din sa pangyayari ang apat pang katao. Inaalam pa ng pulisya ang motibo sa pamamaslang.</t>
         </is>
       </c>
       <c r="C796" s="4" t="inlineStr">
@@ -21157,7 +21157,7 @@
       </c>
       <c r="B828" s="5" t="inlineStr">
         <is>
-          <t>Gayunman, hinimok ng PHLPost ang publiko na bumibili online na isumite ang kanilang mga stamp order sa Pinoy eMall site upang makabili sa aktuwal na presyo. "Upang protektahan ang interes ng publiko, hinihikayat namin ang lahat na magkaroon ng bahagi sa Pope Francis memorabilia sa pamamagitan ng mga selyo na mabibili online sa pamamagitan ng PHLPost web portal, at face value," sabi ni Postmaster General Josie Dela Cruz. Ito ang naging panawagan ng PHLPost kasunod ng mga ulat na ibinebenta sa black market ang mga kopya ng nasabing commemorative stamp nang doble sa aktuwal na presyo nito. Upang makabili ng mga stamp, mag-log on sa www.phlpost.gov.ph at i-click ang Pinoy eMall na magbubukas sa website na Pinoy e-Mall.</t>
+          <t>Gayunman, hinimok ng PHLPost ang publiko na bumibili online na isumite ang kanilang mga stamp order sa Pinoy eMall site upang makabili sa aktuwal na presyo. "Upang protektahan ang interes ng publiko, hinihikayat namin ang lahat na magkaroon ng bahagi sa Pope Francis memorabilia sa pamamagitan ng mga selyo na mabibili online sa pamamagitan ng PHLPost web portal, at face value," sabi ni Postmaster General Josie Dela Cruz. Ito ang naging panawagan ng PHLPost kasunod ng mga ulat na ibinebenta sa black market ang mga kopya ng nasabing commemorative stamp nang doble sa aktuwal na presyo nito. Upang makabili ng mga stamp, mag-log on sa at i-click ang Pinoy eMall na magbubukas sa website na Pinoy e-Mall.</t>
         </is>
       </c>
       <c r="C828" s="4" t="inlineStr">
@@ -21982,7 +21982,7 @@
       </c>
       <c r="B861" s="5" t="inlineStr">
         <is>
-          <t>Ang Bagong Taon ay isang maginhawang pagsisimula, isang pag-aasam, na may mga paghahangad para sa mabuting taon. Karaniwang sinasalubong ang Bagong Taon sa kasiyahan, street dancing, at mga party sa Bisperas ng Bagong Taon. Lumilikha ng ingay at sinisindihan ang mga kuwitis at paputok, upang palayasin ang luma at salubungin ang bagong taon sa pamamagitan ng pagkakapit-bisig at pag-awit ng "Auld Lang Syne". Sinasalubong ng mga Pilipino ang Bagong Taon ng may mga paputok, paghahampas ng mga kaserola, pagbubusina ng mga sasakyan, at pag-aalog ng mga barya, na pinaniniwalaang nagtataboy ng masasamang espiritu at pumipigil sa pagpasok ng kamalasan sa Bagong Taon. May piging sa mga hapagkainan bilang Media Noche, noodles para sa mahabang buhay, at 12 bilugang prutas para sa mabuting kalusugan at magandang kapalaran para sa susunod na 12 buwan. Ang tradisyonal na simbolo ng New Year's Day ay isang sanggol na lalaki (tinatawag na Baby Boy New Year) na may sash kung saan nakasulat ang bagong taon. Sa pagtatapos ng taon siya ay isa nang matanda (tinatawag na Father Time o Old Year) na may sash kung saan nakasulat ang nagdaang taon na ipinapasa ang kanyang tungkulin sa susunod na sanggol ng Bagong Taon.</t>
+          <t>Ang Bagong Taon ay isang maginhawang pagsisimula, isang pag-aasam, na may mga paghahangad para sa mabuting taon. Karaniwang sinasalubong ang Bagong Taon sa kasiyahan, street dancing, at mga party sa Bisperas ng Bagong Taon. Lumilikha ng ingay at sinisindihan ang mga kuwitis at paputok, upang palayasin ang luma at salubungin ang bagong taon sa pamamagitan ng pagkakapit-bisig at pag-awit ng "Auld Lang Syne". Sinasalubong ng mga Pilipino ang Bagong Taon ng may mga paputok, paghahampas ng mga kaserola, pagbubusina ng mga sasakyan, at pag-aalog ng mga barya, na pinaniniwalaang nagtataboy ng masasamang espiritu at pumipigil sa pagpasok ng kamalasan sa Bagong Taon. May piging sa mga hapagkainan bilang Media Noche, noodles para sa mahabang buhay, at 12 bilugang prutas para sa mabuting kalusugan at magandang kapalaran para sa susunod na 12 buwan. Ang tradisyonal na simbolo ng New Year's Day ay isang sanggol na lalaki (tinatawag na Ba ) na may sash kung saan nakasulat ang bagong taon. Sa pagtatapos ng taon siya ay isa nang matanda (tinatawag na Father Time o Old Year) na may sash kung saan nakasulat ang nagdaang taon na ipinapasa ang kanyang tungkulin sa susunod na sanggol ng Bagong Taon.</t>
         </is>
       </c>
       <c r="C861" s="4" t="inlineStr">
@@ -22107,7 +22107,7 @@
       </c>
       <c r="B866" s="5" t="inlineStr">
         <is>
-          <t>Sinabi pa ng dating pangulo na hindi niya kailanman maaaring ipag-utos na ipapatay si Dacer dahil kumpare niya ito. "Nagpapasalamat ako at naliwanagan ang isip niya at nagsasabi siya ng pawang katotohanan," ani Erap. "Alam n'yo, si Bubby Dacer ay parang magkapatid po kami niyan. Inaanak ko iyung anak niya sa binyag. Hanggang ikinasal, ako pa rin ang ninong. Proud [ako] sa pagkakaibigan namin niyan. Imposibleng mangyari sa akin na ako makasali d'yan," pahayag ni Estrada. Pinayuhan naman nito si Mancao na harapin nito ang paratang laban sa kanya. Paliwanag ni Erap, kung walang kasalanan si Mancao ay tiyak na malilinis niya ang kanyang pangalan. Ang mensahe ni Erap ay kasunod nang pagpapahayag si Mancao nang kagustuhan sumuko mula sa dalawang taong pagtatago sa kamay ng batas matapos na tumakas mula sa National Bureau of Investigation (NBI) noong 2013, isang araw bago siya ilipat sa Manila City Jail, dahil umano sa mga banta sa kanyang buhay.</t>
+          <t>Sinabi pa ng dating pangulo na hindi niya kailanman maaaring ipag-utos na ipapatay si Dacer dahil kumpare niya ito. "Nagpapasalamat ako at naliwanagan ang isip niya at nagsasabi siya ng pawang katotohanan," ani Erap. "Alam n'yo, si Bub Inaanak ko iyung anak niya sa binyag. Hanggang ikinasal, ako pa rin ang ninong. Proud [ako] sa pagkakaibigan namin niyan. Imposibleng mangyari sa akin na ako makasali d'yan," pahayag ni Estrada. Pinayuhan naman nito si Mancao na harapin nito ang paratang laban sa kanya. Paliwanag ni Erap, kung walang kasalanan si Mancao ay tiyak na malilinis niya ang kanyang pangalan. Ang mensahe ni Erap ay kasunod nang pagpapahayag si Mancao nang kagustuhan sumuko mula sa dalawang taong pagtatago sa kamay ng batas matapos na tumakas mula sa National Bureau of Investigation (NBI) noong 2013, isang araw bago siya ilipat sa Manila City Jail, dahil umano sa mga banta sa kanyang buhay.</t>
         </is>
       </c>
       <c r="C866" s="4" t="inlineStr">
@@ -23607,7 +23607,7 @@
       </c>
       <c r="B926" s="7" t="inlineStr">
         <is>
-          <t>Sa unang pagkakataon, napanood ng publiko ang digitally restored at remastered na mga kopya ng Anak directed by Rory Quintos, Kapag Langit ang Humatol directed by Laurice Guillen at Bata, Bata, Paano ka Ginawa ni Chito Rono. Mabusising inayos, pinalinaw at pinaganda ng ABS-CBN Film Archives at Central Digita Labs ang naturang mga pelikula. Dumating ang ilang ABS-CBN executives at director na kinabibilangan nina Ms. Malou Santos, Chit Guerrero, Olive Lamasan, Rory Quintos, Laurice Guillen at Chito Rono sa UP Film Center para panoorin ang Bata, Bata.... Dumating din sina Cherrie Pie Picache at Albert Martinez, na kasama sa cast nito. In full force din na dumating sa event ang Vilmanians at press people. Sa totoo lang, aakalain mong bago ang kopya ng restored films. Kung hindi nga lang naroroon sina Carlo Aquino at Serena Dalrymple na mga totoy at nene pa ang itsura sa movie, aakalain mong bagong pelikula ang Bata... Bata.... Salamat sa modernong teknolohiya. Sabi sa speech ni Leo Katigbak, ang ABS-CBN Film Archives head, anim nang classic film ni Ate Vi ang na-restore nila at baka nga lumobo pa ito sa maraming kopya dahil sa magandang pagtanggap ng publiko. Sa talumpati naman ni Ate Vi, aniyang pabiro, "Anim pa lang? Bakit hindi 15?" At idinagdag na, "Modesty aside, marami tayong classic films na nagawa na kailangan munang i-restore dahil sa kalumaan." "Gusto naming i-restore ang mga natatanging pelikula ni Vilma mula sa iba't ibang direktor," kuwento pa ni Mr. Katigbak. All in all, nakapag-restore na ang ABS-CBN Film Archives ng 72 pelikula since 2011 at ang ilan sa mga ito ay pinalad na maipalabas sa international filmfest at sa katunayan ay may red-carpet pang premiere na naganap at naiere sa free-to-air/cable television. Napapanood din ang mga ito sa pay-per-view at video-on-demand, nabibili sa DVD at nada-download din sa iTunes. Sa tanong kay Ate Vi kung ano pa ang nagawa niyang pelikula na gusto niyang panoorin, ang excited niyang sagot, "T-Bird at Ako."</t>
+          <t>Sa unang pagkakataon, napanood ng publiko ang digitally restored at remastered na mga kopya ng Anak directed , Kapag Langit ang Humatol directed , Bata, Paano ka Ginawa ni Chito Rono. Mabusising inayos, pinalinaw at pinaganda ng ABS-CBN Film Archives at Central Digita Labs ang naturang mga pelikula. Dumating ang ilang ABS-CBN executives at director na kinabibilangan nina Ms. Malou Santos, Chit Guerrero, Olive Lamasan, Rory Quintos, Laurice Guillen at Chito Rono sa UP Film Center para panoorin ang Bata, Bata.... Dumating din sina Cherrie Pie Picache at Albert Martinez, na kasama sa cast nito. In full force din na dumating sa event ang Vilmanians at press people. Sa totoo lang, aakalain mong bago ang kopya ng restored films. Kung hindi nga lang naroroon sina Carlo Aquino at Serena Dalrymple na mga totoy at nene pa ang itsura sa movie, aakalain mong bagong pelikula ang Bata... Bata.... Salamat sa modernong teknolohiya. Sabi sa speech ni Leo Katigbak, ang ABS-CBN Film Archives head, anim nang classic film ni Ate Vi ang na-restore nila at baka nga lumobo pa ito sa maraming kopya dahil sa magandang pagtanggap ng publiko. Sa talumpati naman ni Ate Vi, aniyang pabiro, "Anim pa lang? Bakit hindi 15?" At idinagdag na, "Modesty aside, marami tayong classic films na nagawa na kailangan munang i-restore dahil sa kalumaan." "Gusto naming i-restore ang mga natatanging pelikula ni Vilma mula sa iba't ibang direktor," kuwento pa ni Mr. Katigbak. All in all, nakapag-restore na ang ABS-CBN Film Archives ng 72 pelikula since 2011 at ang ilan sa mga ito ay pinalad na maipalabas sa international filmfest at sa katunayan ay may red-carpet pang premiere na naganap at naiere sa free-to-air/cable television. Napapanood din ang mga ito sa pay-per-view at video-on-demand, nabibili sa DVD at nada-download din sa iTunes. Sa tanong kay Ate Vi kung ano pa ang nagawa niyang pelikula na gusto niyang panoorin, ang excited niyang sagot, "T-Bird at Ako."</t>
         </is>
       </c>
       <c r="C926" s="6" t="inlineStr">
@@ -23657,7 +23657,7 @@
       </c>
       <c r="B928" s="7" t="inlineStr">
         <is>
-          <t>Mainit na tinanggap si Willie ng Kapuso Network sa pangunguna ni GMA Network Chairman/CEO Atty. Felipe L. Gozon na nagsabing, "We are pleased to have Willie Revillame's program in the network. Willie has a very large following. Through our partnership with WBR Entertainment, GMA Network will be a part of the long awaited return of Willie Revillame on television." "We are very grateful and glad to have our program Wowowin shown in GMA Network, the number one TV station in the country. We will see to it that we deserve the trust reposed on us by GMA Network," sabi naman ni Willie. Kilalang "overtime king" si Willie dahil mahilig mag-overtime ng kanyang show, naaapektuhan tuloy ang airing time ng kasunod niyang show. Nangyari ito sa ABS-CBN noon at naulit sa TV5. Nabanggit ito ng ilang press people sa isang bossing ng GMA-7, pero ang sagot nito, ipaaalala nila kay Willie na 'pag mag-overtime siya, puputulin ang kanyang show, kaya kailangan niyang sumunod sa oras. Kapag mapuputol ang show niya, hindi siya dapat magtampo dahil sinusunod lang ng network ang airing time ng shows nila. Noon pa nabalitaan na sina Mike Enriquez at Joey de Leon ang tumulong para makapasok si Willie sa GMA-7. Samantala, isa ang pangalan ni Jennylyn Mercado sa nabanggit ng spy namin na magiging co-host ni Willie Revillame sa Wowowin. Ni-request daw ang aktres na maging co-host , hindi lang malinaw kung si Willie mismo o ang staff niya ang nag-request sa management ng network. Kung matutuloy sa show ni Willie si Jennylyn, magiging dalawa ang show niya pagkatapos ng drama series niyang Second Chances. Isa rin siya sa three judges ng nagbabalik na Starstruck kasama sina Joey de Leon at Regine Velasquez. May experience na sa hosting si Jennylyn dahil naging host siya sa reality show na Anak Ko 'To at sa Showbiz Central and in fairness, kaya ng power niyang mag-host. Pansamantala, nagpapakaaktres muna siya sa Second Chances na may mainit na talakayan sa social media kung kanino mas nababagay ang karakter ni Jennylyn na si Lyra -- kay Bernard (Raymart Santiago) o kay Jerome (Rafael Rosell).</t>
+          <t>Mainit na tinanggap si Willie ng Kapuso Network sa pangunguna ni GMA Network Chairman/CEO Atty. Felipe L. Gozon na nagsabing, "We are pleased to have Willie Revillame's program in the network. Willie has a very large following. Through our partnership with WBR Entertainment, GMA Network will be a part of the long awaited return of Willie Revillame on television." "We are very grateful and glad to have our program Wowowin shown in GMA Network, the number one TV station in the country. We will see to it that we deserve the trust reposed on us ," sabi naman ni Willie. Kilalang "overtime king" si Willie dahil mahilig mag-overtime ng kanyang show, naaapektuhan tuloy ang airing time ng kasunod niyang show. Nangyari ito sa ABS-CBN noon at naulit sa TV5. Nabanggit ito ng ilang press people sa isang bossing ng GMA-7, pero ang sagot nito, ipaaalala nila kay Willie na 'pag mag-overtime siya, puputulin ang kanyang show, kaya kailangan niyang sumunod sa oras. Kapag mapuputol ang show niya, hindi siya dapat magtampo dahil sinusunod lang ng network ang airing time ng shows nila. Noon pa nabalitaan na sina Mike Enriquez at Joey de Leon ang tumulong para makapasok si Willie sa GMA-7. Samantala, isa ang pangalan ni Jennylyn Mercado sa nabanggit ng spy namin na magiging co-host ni Willie Revillame sa Wowowin. Ni-request daw ang aktres na maging co-host , hindi lang malinaw kung si Willie mismo o ang staff niya ang nag-request sa management ng network. Kung matutuloy sa show ni Willie si Jennylyn, magiging dalawa ang show niya pagkatapos ng drama series niyang Second Chances. Isa rin siya sa three judges ng nagbabalik na Starstruck kasama sina Joey de Leon at Regine Velasquez. May experience na sa hosting si Jennylyn dahil naging host siya sa reality show na Anak Ko 'To at sa Showbiz Central and in fairness, kaya ng power niyang mag-host. Pansamantala, nagpapakaaktres muna siya sa Second Chances na may mainit na talakayan sa social media kung kanino mas nababagay ang karakter ni Jennylyn na si Lyra -- kay Bernard (Raymart Santiago) o kay Jerome (Rafael Rosell).</t>
         </is>
       </c>
       <c r="C928" s="6" t="inlineStr">
@@ -23982,7 +23982,7 @@
       </c>
       <c r="B941" s="7" t="inlineStr">
         <is>
-          <t>Kaya naman masaya siya, at aminadong feeling leading man na, nang dumating siya sa second presscon niya for that day nitong Martes. Una ang presscon nila ng leading lady niyang si Valeen Montenegro para sa movie nilang The Write Moment, na ipalalabas na, produced by IdeaFirst Company at Viva Entertainment. Ipinalabas na last year ang nasabing pelikula sa Quezon City Film Festival. Kuwento ni Jerald, sa movie ay gagampanan niya ang karakter ni Dave, isang professional wedding videographer na sideline ang pagiging movie scriptwriter. Girlfriend niya si Valeen, as Joyce, na bigla na lamang siyang hiniwalayan nang walang dahilan. Hindi niya matanggap iyon, kaya naman napasulat tuloy sila ng movie script para sa kanilang dalawa ni Joyce, ang kaibahan, happy ang ending ng isinulat niyang story. Sa huli, na-realize niya na kailangan lang pala niyang sundin ang sarili niyang script para magkatuluyan sila. Ang daming hugot lines sa movie na tiyak na magugustuhan ng mga manonood. Sa direksiyon ni Dominic Lim, showing na ang The Write Moment sa Wednesday, June 27, in cinemas nationwide. May premiere night sila sa Monday, June 25, sa Robinson's Galleria. "Sa palagay ko po, sa The Write Moment ay nabuksan ang doors sa akin, na puwede pala akong maging leading man," biro ni Jerald. "Kaya very thankful po ako na in-accept nila ako, na from drama sa theatre, nagpapatawa ako. At kita poi to sa live audience sa Sunday Pinasaya ng GMA-7. "May gagawin din akong three movies, ang Nakalimutan Kong Kalimutan Ka with Alex Gonzaga at Vin Abrenica; Pangarap kong Holdup with Paolo Contis; at Mina Anod with Dennis Trillo. "Sa Real, Quezon kami magsu-shoot (ni Dennis), dahil tungkol sa surfing ang story nito. Sa August po ay mapapanood na rin ako sa Rak of Aegis sa PETA, sa third year na presentation nito." Kumusta naman ang love life ni Jerald, may gusto ba talaga siya kay Valeen? "Hindi po totoo, kulitan lang naming 'yun ni Valeen sa Sunday Pinasaya. Nagkikita pa rin kami ng French girlfriend ko, like noong minsang dumating siya, kasama ang boyfriend niya," kuwento pa ni Jerald. "Dati ay pinasusunod niya ako sa France, pero hindi ko ginawa. Sayang naman 'yung career ko rito, na medyo bumobongga na ngayon. "Mas gusto kong mabigyan muna ng magandang buhay ang pamilya ko. Gusto kong mabigyan ng bahay ang nanay ko at maipasyal siya sa ibang bansa kapag nakaipon pa ako," seryoso nang sabi ni Jerald.</t>
+          <t>Kaya naman masaya siya, at aminadong feeling leading man na, nang dumating siya sa second presscon niya for that day nitong Martes. Una ang presscon nila ng leading lady niyang si Valeen Montenegro para sa movie nilang The Write Moment, na ipalalabas na, produced Ipinalabas na last year ang nasabing pelikula sa Quezon City Film Festival. Kuwento ni Jerald, sa movie ay gagampanan niya ang karakter ni Dave, isang professional wedding videographer na sideline ang pagiging movie scriptwriter. Girlfriend niya si Valeen, as Joyce, na bigla na lamang siyang hiniwalayan nang walang dahilan. Hindi niya matanggap iyon, kaya naman napasulat tuloy sila ng movie script para sa kanilang dalawa ni Joyce, ang kaibahan, happy ang ending ng isinulat niyang story. Sa huli, na-realize niya na kailangan lang pala niyang sundin ang sarili niyang script para magkatuluyan sila. Ang daming hugot lines sa movie na tiyak na magugustuhan ng mga manonood. Sa direksiyon ni Dominic Lim, showing na ang The Write Moment sa Wednesday, June 27, in cinemas nationwide. May premiere night sila sa Monday, June 25, sa Robinson's Galleria. "Sa palagay ko po, sa The Write Moment ay nabuksan ang doors sa akin, na puwede pala akong maging leading man," biro ni Jerald. "Kaya very thankful po ako na in-accept nila ako, na from drama sa theatre, nagpapatawa ako. At kita poi to sa live audience sa Sunday Pinasaya ng GMA-7. "May gagawin din akong three movies, ang Nakalimutan Kong Kalimutan Ka with Alex Gonzaga at Vin Abrenica; Pangarap kong Holdup with Paolo Contis; at Mina Anod with Dennis Trillo. "Sa Real, Quezon kami magsu-shoot (ni Dennis), dahil tungkol sa surfing ang story nito. Sa August po ay mapapanood na rin ako sa Rak of Aegis sa PETA, sa third year na presentation nito." Kumusta naman ang love life ni Jerald, may gusto ba talaga siya kay Valeen? "Hindi po totoo, kulitan lang naming 'yun ni Valeen sa Sunday Pinasaya. Nagkikita pa rin kami ng French girlfriend ko, like noong minsang dumating siya, kasama ang boyfriend niya," kuwento pa ni Jerald. "Dati ay pinasusunod niya ako sa France, pero hindi ko ginawa. Sayang naman 'yung career ko rito, na medyo bumobongga na ngayon. "Mas gusto kong mabigyan muna ng magandang buhay ang pamilya ko. Gusto kong mabigyan ng bahay ang nanay ko at maipasyal siya sa ibang bansa kapag nakaipon pa ako," seryoso nang sabi ni Jerald.</t>
         </is>
       </c>
       <c r="C941" s="6" t="inlineStr">
@@ -24057,7 +24057,7 @@
       </c>
       <c r="B944" s="7" t="inlineStr">
         <is>
-          <t>"He is the FATHER you thought you knew. The Cosby Show was my today's tv reality show. Thank you. That's all I would like to say :)," pahayag ni Evin, 38.</t>
+          <t>"He is the FATHER you thought you knew. The Cos 's tv reality show. Thank you. That's all I would like to say :)," pahayag ni Evin, 38.</t>
         </is>
       </c>
       <c r="C944" s="6" t="inlineStr">
@@ -25132,7 +25132,7 @@
       </c>
       <c r="B987" s="7" t="inlineStr">
         <is>
-          <t>NIYANIG ng magnitude 4.5 lindol ang Surigao del Norte kaninang umaga. Ayon sa Philippine Institute of Volcanology and Seismology ang pagyanig na ito ay aftershock ng magnitude 5.9 lindol sa Surigao del Norte noong Pebrero 8.  Naramdaman ang lindol alas-11:06 ng umaga. Ang epicenter nito ay 47 kilometro sa silangan ng General Luna. May lalim itong anim na kilometro at sanhi ng paggalaw ng tectonic plate. Nagresulta ito sa Intensity IV paggalaw sa General Luna.</t>
+          <t>NIYANIG ng magnitude 4.5 lindol ang Surigao del Norte kaninang umaga. Ayon sa Philippine Institute of Volcanology and Seismology ang pagyanig na ito ay aftershock ng magnitude 5.9 lindol sa Surigao del Norte noong Pebrero 8. Naramdaman ang lindol alas-11:06 ng umaga. Ang epicenter nito ay 47 kilometro sa silangan ng General Luna. May lalim itong anim na kilometro at sanhi ng paggalaw ng tectonic plate. Nagresulta ito sa Intensity IV paggalaw sa General Luna.</t>
         </is>
       </c>
       <c r="C987" s="6" t="inlineStr">
@@ -25807,7 +25807,7 @@
       </c>
       <c r="B1014" s="7" t="inlineStr">
         <is>
-          <t>SA halip na suwertehin, baka malasin ang iyong New Year dahil sa mga pampasuwerte na may sangkap ng cadmium at lead. Ayon sa EcoWaste Coalition nagsagawa ito ng pagsusuri sa mga lucky charm na mabenta ngayong Chinese New Year of the Earth Pig. Bumili ito ng 20 piraso ng lucky charm na nagkakahalaga ng P25-P300 bawat isa sa Binondo at Quiapo at sinuri ito gamit ang X-Ray Fluorescence analytical instrument.  "Some lucky charms and amulets that are supposed to attract energy, health, fortune and happiness are unluckily contaminated with cadmium and lead, two highly hazardous substances that belong to the WHO's list of 10 chemicals of major public health concern," ani Thony Dizon, Chemical Safety Campaigner ng EcoWaste. Sa mga sinuri, 15 ang mayroong lead at cadmium na lagpas sa pinapayagan ng batas ng bansa, sa Estados Unidos at European Union. "Cadmium and lead, which can accumulate in the body and damage human health, should not be present in consumer products, especially for items that are supposed to enhance good health and better life," ani Dizon.</t>
+          <t>SA halip na suwertehin, baka malasin ang iyong New Year dahil sa mga pampasuwerte na may sangkap ng cadmium at lead. Ayon sa EcoWaste Coalition nagsagawa ito ng pagsusuri sa mga lucky charm na mabenta ngayong Chinese New Year of the Earth Pig. Bumili ito ng 20 piraso ng lucky charm na nagkakahalaga ng P25-P300 bawat isa sa Binondo at Quiapo at sinuri ito gamit ang X-Ray Fluorescence analytical instrument. "Some lucky charms and amulets that are supposed to attract energy, health, fortune and happiness are unluckily contaminated with cadmium and lead, two highly hazardous substances that belong to the WHO's list of 10 chemicals of major public health concern," ani Thony Dizon, Chemical Safety Campaigner ng EcoWaste. Sa mga sinuri, 15 ang mayroong lead at cadmium na lagpas sa pinapayagan ng batas ng bansa, sa Estados Unidos at European Union. "Cadmium and lead, which can accumulate in the body and damage human health, should not be present in consumer products, especially for items that are supposed to enhance good health and better life," ani Dizon.</t>
         </is>
       </c>
       <c r="C1014" s="6" t="inlineStr">
@@ -26482,7 +26482,7 @@
       </c>
       <c r="B1041" s="7" t="inlineStr">
         <is>
-          <t>Sa pulong balitaan kahapon ng tanghali sa kanyang tahanan, nanindigan si Gomez na bababa lamang siya sa puwesto pagkatapos ng kanyang termino sa Hunyo 2019. Ayon kay Gomez, hindi niya tatanggapin ang naturang recall election na inihain laban sa kanya ng mga tagasuporta ni dating San Juan Vice Mayor Francis Zamora, at inaprubahan ng Commission on Elections (Comelec), dahil paano umano mawawalan ng tiwala sa kanya ang kanyang constituents gayong napakarami niyang proyekto at dalawang magkasunod na taon (2016 at 2017) pa nakatanggap ng Seal of Good Governance award mula sa Department of Interior and Local Government (DILG) ang San Juan. Tiniyak din ni Gomez na iaapela nila ang naturang desisyon ng poll body sa legal na paraan at naaayon sa tamang proseso. "I will not accept this recall and will allow my lawyers to challenge it legally and according to the right process," ani Gomez. "The recall petition castrated by Francis Zamora, is not the true will of the people of San Juan. It is the project of their machinations. I will not allow myself to fall in his ill motives." Pinayuhan din ni Gomez si Zamora na maghintay na lamang na matapos ang kanyang panunungkulan dahil hindi na siya muling tatakbo sa susunod na eleksiyon, dahil ito na ang kanyang ikatlo at huling termino bilang alkalde ng San Juan. "I will step down as mayor of San Juan in June 30, 2019 as I finish my term in 18-months. Ewan ko ba kung bakit di pa siya (Zamora) makapaghintay," aniya pa. Pinabulaanan din ni Gomez ang akusasyon ni Zamora na nagtatago siya at hindi pumapasok sa kanyang opisina upang iwasang matanggap ang notice of sufficiency ng Comelec kaugnay ng recall election. Gayunman, aminado ang alkalde na wala siyang planong tanggapin ang naturang notice of sufficiency, dahil kailangan muna niya itong ikonsulta sa kanyang abogado. Yes! Dedma lang po dapat, cuz for us, Z is DEAD..hahaahahahhaarsh.. such a cry baby boy. no need to do recall. fake nman mga signatures..also fake naman ung mga scholarships &amp; medical assistance. alam nya nman talgang walang mapupuntahan petition nya. makulit lang siya, kala nya mababali nya batas. lol wag kasing assuming Sir Francis.napahiya ka tuloy. hahaha, kung ako sau paghandaan mo ung mga pakulo mong medical assistance at scholarships. Karma lang tlga sasalubong sau.</t>
+          <t>Sa pulong balitaan kahapon ng tanghali sa kanyang tahanan, nanindigan si Gomez na bababa lamang siya sa puwesto pagkatapos ng kanyang termino sa Hunyo 2019. Ayon kay Gomez, hindi niya tatanggapin ang naturang recall election na inihain laban sa kanya ng mga tagasuporta ni dating San Juan Vice Mayor Francis Zamora, at inaprubahan ng Commission on Elections (Comelec), dahil paano umano mawawalan ng tiwala sa kanya ang kanyang constituents gayong napakarami niyang proyekto at dalawang magkasunod na taon (2016 at 2017) pa nakatanggap ng Seal of Good Governance award mula sa Department of Interior and Local Government (DILG) ang San Juan. Tiniyak din ni Gomez na iaapela nila ang naturang desisyon ng poll body sa legal na paraan at naaayon sa tamang proseso. "I will not accept this recall and will allow my lawyers to challenge it legally and according to the right process," ani Gomez. "The recall petition castrated , is not the true will of the people of San Juan. It is the project of their machinations. I will not allow myself to fall in his ill motives." Pinayuhan din ni Gomez si Zamora na maghintay na lamang na matapos ang kanyang panunungkulan dahil hindi na siya muling tatakbo sa susunod na eleksiyon, dahil ito na ang kanyang ikatlo at huling termino bilang alkalde ng San Juan. "I will step down as mayor of San Juan in June 30, 2019 as I finish my term in 18-months. Ewan ko ba kung bakit di pa siya (Zamora) makapaghintay," aniya pa. Pinabulaanan din ni Gomez ang akusasyon ni Zamora na nagtatago siya at hindi pumapasok sa kanyang opisina upang iwasang matanggap ang notice of sufficiency ng Comelec kaugnay ng recall election. Gayunman, aminado ang alkalde na wala siyang planong tanggapin ang naturang notice of sufficiency, dahil kailangan muna niya itong ikonsulta sa kanyang abogado. Yes! Dedma lang po dapat, cuz for us, Z is DEAD..hahaahahahhaarsh.. such a cry baby boy. no need to do recall. fake nman mga signatures..also fake naman ung mga scholarships &amp; medical assistance. alam nya nman talgang walang mapupuntahan petition nya. makulit lang siya, kala nya mababali nya batas. lol wag kasing assuming Sir Francis.napahiya ka tuloy. hahaha, kung ako sau paghandaan mo ung mga pakulo mong medical assistance at scholarships. Karma lang tlga sasalubong sau.</t>
         </is>
       </c>
       <c r="C1041" s="6" t="inlineStr">
@@ -26932,7 +26932,7 @@
       </c>
       <c r="B1059" s="7" t="inlineStr">
         <is>
-          <t>INIHAYAG ni dating Presidential Spokesperson Harry Roque ang kanyang pag-atras sa kanyang kandidatura sa pagka-senador dahil sa isyu sa kanyang kalusugan.  "It is with a truly heavy heart that I announce the withdrawal of my senatorial bid. I have recently undergone a percutaneous coronary intervention following the discovery of an unstable angina coronary disease earlier this week. In the days since the procedure, my family and I have been forced to confront the reality of my physical situation and what it ultimately means for my aspirations to public service," sabi ni Roque sa isang pahayag.  Kasabay nito, nagpasalamat si Roque sa mga sumuporta sa kanyang planong pagtakbo sa Senado. "I wish to thank all who have been so kind and supportive of my candidacy. I ran for senator because I wanted to be of service in a way that I know I will be highly effective. Whatever they may think of my politics, those who have seen my work in both the public and private sector can attest to what I would have brought to the Senate. Unfortunately, for the moment, it seems that God has other plans," ayon pa kay Roque.  Umaasa naman si Roque na makakapagserbisyo siya muli sa publiko. "It is my sincere hope that I will someday again have the honor to serve the Filipino people as a legislator, or in whatever other capacity I may be of service. I continue to support our President and this administration and wish only the best for our country. God bless us all!" dagdag ni Roque. Nagpaabot naman ng mensahe si Presidential Spokesperson at Chief Presidential Legal Counsel Salvador Panelo kay Roque.  "I personally wish him good health," sabi ni Panelo.</t>
+          <t>INIHAYAG ni dating Presidential Spokesperson Harry Roque ang kanyang pag-atras sa kanyang kandidatura sa pagka-senador dahil sa isyu sa kanyang kalusugan. "It is with a truly heavy heart that I announce the withdrawal of my senatorial bid. I have recently undergone a percutaneous coronary intervention following the discovery of an unstable angina coronary disease earlier this week. In the days since the procedure, my family and I have been forced to confront the reality of my physical situation and what it ultimately means for my aspirations to public service," sabi ni Roque sa isang pahayag. Kasabay nito, nagpasalamat si Roque sa mga sumuporta sa kanyang planong pagtakbo sa Senado. "I wish to thank all who have been so kind and supportive of my candidacy. I ran for senator because I wanted to be of service in a way that I know I will be highly effective. Whatever they may think of my politics, those who have seen my work in both the public and private sector can attest to what I would have brought to the Senate. Unfortunately, for the moment, it seems that God has other plans," ayon pa kay Roque. Umaasa naman si Roque na makakapagserbisyo siya muli sa publiko. "It is my sincere hope that I will someday again have the honor to serve the Filipino people as a legislator, or in whatever other capacity I may be of service. I continue to support our President and this administration and wish only the best for our country. God bless us all!" dagdag ni Roque. Nagpaabot naman ng mensahe si Presidential Spokesperson at Chief Presidential Legal Counsel Salvador Panelo kay Roque. "I personally wish him good health," sabi ni Panelo.</t>
         </is>
       </c>
       <c r="C1059" s="6" t="inlineStr">
@@ -27057,7 +27057,7 @@
       </c>
       <c r="B1064" s="7" t="inlineStr">
         <is>
-          <t>UMAABOT sa 240 Filipino ang namamatay araw-araw sa mga smoking related diseases. Kaya kung papatawan ang sigarilyo ng P90 bawat kaha ay maraming buhay ang maililigtas. Ayon sa HealthJustice Philippines mababawasan ng 1 milyon ang mga naninigarilyo sa 2022 kapag natuloy ang pagtataas sa buwis na ipinapataw sa sigarilyo na nangangahulugan na mas marami ang maililigtas. "We are expectant that our champions in health will approve the raise in excise tax to 90 pesos to effectively curb smoking among Filipinos and to help fund the UHC that is set to be signed by anytime now," ani Mary Ann Mendoza, pangulo ng HealthJustice Philippines. Ayon sa cancer survivor na si Engr. Emer Rojas, pangulo ng New Vois Association of the Philippines, bumababa ang bilang ng mga naninigarilyo kapag mataas ang buwis nito. "It is our responsibility to help the next generation to live in a smoke-free environment. 240 Filipinos die every day because of smoking re-related diseases in the Philippines. We urge our senators to fast track the deliberations on the tobacco tax bills because the health of the Filipinos is at stake here," ani Rojas. Umaasa ang HealthJustice Philippines na maipapasa ng Senado ang panukala bago mag-adjourn ang sesyon sa Biyernes. "We are hopeful that the committee on Ways and Means headed by Senator Sonny Angara will pass the further increase in excise tax on tobacco before the Congress will go on break on February 9, considering that President Rodrigo Duterte has recently certified the increase in tobacco tax bills as urgent," dagdag pa ni Mendoza. Sa pagdinig noong Enero 29 ay nabigo ang Senate Ways and Means committee na pinamumunuan ni Sen. Sonny Angara na aprubahan ang committee report na ipadadala sa plenaryo upang pagbotohan sa ikalawa at ikatlong pagbasa. Bukod sa mababawasan ang mga nagkakasakit dahil sa sigarilyo, ang pondo na kikitain sa dagdag na buwis ay gagamitin upang punan ang kakulangan sa pagpapatupad ng Universal Health Care Act. Kakailanganin ng P257 bilyon sa implementasyon ng UHC subalit ang DOH, PhilHealth, PCSO, at PAGCOR ay mayroon lamang P217 bilyon.</t>
+          <t>UMAABOT sa 240 Filipino ang namamatay araw-araw sa mga smoking related diseases. Kaya kung papatawan ang sigarilyo ng P90 bawat kaha ay maraming buhay ang maililigtas. Ayon sa HealthJustice Philippines mababawasan ng 1 milyon ang mga naninigarilyo sa 2022 kapag natuloy ang pagtataas sa buwis na ipinapataw sa sigarilyo na nangangahulugan na mas marami ang maililigtas. "We are expectant that our champions in health will approve the raise in excise tax to 90 pesos to effectively curb smoking among Filipinos and to help fund the UHC that is set to be signed by anytime now," ani Mary Ann Mendoza, pangulo ng HealthJustice Philippines. Ayon sa cancer survivor na si Engr. Emer Rojas, pangulo ng New Vois Association of the Philippines, bumababa ang bilang ng mga naninigarilyo kapag mataas ang buwis nito. "It is our responsibility to help the next generation to live in a smoke-free environment. 240 Filipinos die every day because of smoking re-related diseases in the Philippines. We urge our senators to fast track the deliberations on the tobacco tax bills because the health of the Filipinos is at stake here," ani Rojas. Umaasa ang HealthJustice Philippines na maipapasa ng Senado ang panukala bago mag-adjourn ang sesyon sa Biyernes. "We are hopeful that the committee on Ways and Means headed r increase in excise tax on tobacco before the Congress will go on break on February 9, considering that President Rodrigo Duterte has recently certified the increase in tobacco tax bills as urgent," dagdag pa ni Mendoza. Sa pagdinig noong Enero 29 ay nabigo ang Senate Ways and Means committee na pinamumunuan ni Sen. Sonny Angara na aprubahan ang committee report na ipadadala sa plenaryo upang pagbotohan sa ikalawa at ikatlong pagbasa. Bukod sa mababawasan ang mga nagkakasakit dahil sa sigarilyo, ang pondo na kikitain sa dagdag na buwis ay gagamitin upang punan ang kakulangan sa pagpapatupad ng Universal Health Care Act. Kakailanganin ng P257 bilyon sa implementasyon ng UHC subalit ang DOH, PhilHealth, PCSO, at PAGCOR ay mayroon lamang P217 bilyon.</t>
         </is>
       </c>
       <c r="C1064" s="6" t="inlineStr">
@@ -27357,7 +27357,7 @@
       </c>
       <c r="B1076" s="7" t="inlineStr">
         <is>
-          <t>Nagsimula nang mag-taping si Dingdong ng Pari 'Koy, ang kanyang bagong inspirational drama series sa GMA-7. First time siyang gaganap bilang pari. Enjoy siya sa taping dahil second time siyang ididirek ni Maryo J. delos Reyes, after ng Pahiram ng Sandali. Makakasama niya sa Pari 'Koy sina Gabby Eigenmann, Sunshine Dizon, Luz Valdez, Chanda Romero, Raymond Bagatsing, JC Tiuseco, Raf Fernanadez, Jeric Gonzales, Hiro Peralta, Diego Castro, Dexter Doria at Jillian Ward at sa March 9 ang premiere telecast nila, bilang kapalit ng matatapos nang More Than Words. Last Monday, nag-judge si Dingdong, as Commissioner of the National Youth Commission, with Sen. Bam Aquino ng Ten Accomplished Youth Organizations (TAYO) Year XII na ginanap sa Senado at Tuesday, ang awarding ng winners na ginanap sa Malacanang. Sunud-sunod naman ang pictorial ni Marian sa mga bago niyang endorsements. Sa Saturday, ilo-launch na siya ng Bench sa kanyang Inner Beauty Scent. Sa March 3 naman ang launch niya as the cover of The New Hair Asia magazine ni Elvie Alvaran. Natapos na rin niya ang pictorial ng isa pa niyang bagong endorsement na malapit na rin ang launch. At basta may free time, sa halip na once a week lamang siya "Juan For All All For Juan" segment ng Eat Bulaga, sinosorpresa niya sina Jose Manalo, Wally Bayola at Paulo Ballesteros kung sa lugar na sinusugod ng mga ito. Nag-taping na rin si Marian ng isang episode para sa Holy Week presentation ng Eat Bulaga. Pinaghahandaan na ring mabuti ni Marian ang bago niyang drama series na The Richman's Daughter (tentative title) na ang story ay tungkol sa family traditions and values. Gaganap siya bilang si Jade, isang magandang babaeng mai-in love sa isa ring wonderful woman. Ayon sa head writer ng soap na si Suzette Doctolero, hindi ito tulad ng My Husband's Lover na una niyang ginawa. Pero ididirek din ito ni Dominic Zapata at makakasama ni Marian sina Luis Alandy, Mike Tan, TJ Trinidad, Glaiza de Castro, Katrina Halili, Glydel Mercado, Al Tantay at si Ms. Gloria Romero. Sa susunod na buwan na magsisimula ang taping nila nito at after Holy Week naman ang airing. Samantala sina Marian at Dingdong ang first guests sa season six ng The Tim Yap Show at maraming kilig moments sa mag-asawa sa mga tanong ni Tim. After the wedding and honeymoon na ang questions like ano ang feeling ngayong mag-asawa na sila? "Nagugulat pa ako kapag tinatawag akong Mrs. Dantes," sagot ni Marian. "At napapangiti ako sa realization na kasal na nga pala ako kay Dingdong." "Napapatigil naman ako kapag nagpi-fill up ako ng document na pagdating sa civil status, napapangiti ako dahil hindi na nga pala ako single," natatawang sagot ni Dingdong. Nakumusta ni Tim ang ama ni Marian na na-meet niya una sa wedding then sa Boracay. "Promise ni Papa, babalik siya muli sa Pilipinas kapag nalamang preggy na ako. Kung sakali, sa akin unang magkakaapo sina Papa at Mama," sabi ng Primetime Queen ng GMA-7. May pangalan na ba silang nakahanda para sa magiging anak nila? "Since Jose Sixto III ako, hindi pa namin alam kung magiging Jose Sixto IV if boy ang magiging anak namin pero kapag girl, laging magkakaroon iyon ng Maria." Simple lang ang wishes ng mag-asawa. Si Dingdong, ayaw niyang mawawalan ng charge ang cellphone niya kaya lagi siyang may dalang powerbank para lagi niyang nakakausap ang esposa. Gusto ni Marian na laging malinis ang kanilang room hanggang banyo kaya siya ang laging naglilinis nito. Hindi siya nagbubukas ng ilaw habang natutulog pa si Dingdong.</t>
+          <t>Nagsimula nang mag-taping si Dingdong ng Pari 'Koy, ang kanyang bagong inspirational drama series sa GMA-7. First time siyang gaganap bilang pari. Enjoy siya sa taping dahil second time siyang ididirek ni Maryo J. delos Reyes, after ng Pahiram ng Sandali. Makakasama niya sa Pari 'Koy sina Gab , Sunshine Dizon, Luz Valdez, Chanda Romero, Raymond Bagatsing, JC Tiuseco, Raf Fernanadez, Jeric Gonzales, Hiro Peralta, Diego Castro, Dexter Doria at Jillian Ward at sa March 9 ang premiere telecast nila, bilang kapalit ng matatapos nang More Than Words. Last Monday, nag-judge si Dingdong, as Commissioner of the National Youth Commission, with Sen. Bam Aquino ng Ten Accomplished Youth Organizations (TAYO) Year XII na ginanap sa Senado at Tuesday, ang awarding ng winners na ginanap sa Malacanang. Sunud-sunod naman ang pictorial ni Marian sa mga bago niyang endorsements. Sa Saturday, ilo-launch na siya ng Bench sa kanyang Inner Beauty Scent. Sa March 3 naman ang launch niya as the cover of The New Hair Asia magazine ni Elvie Alvaran. Natapos na rin niya ang pictorial ng isa pa niyang bagong endorsement na malapit na rin ang launch. At basta may free time, sa halip na once a week lamang siya "Juan For All All For Juan" segment ng Eat Bulaga, sinosorpresa niya sina Jose Manalo, Wally Bayola at Paulo Ballesteros kung sa lugar na sinusugod ng mga ito. Nag-taping na rin si Marian ng isang episode para sa Holy Week presentation ng Eat Bulaga. Pinaghahandaan na ring mabuti ni Marian ang bago niyang drama series na The Richman's Daughter (tentative title) na ang story ay tungkol sa family traditions and values. Gaganap siya bilang si Jade, isang magandang babaeng mai-in love sa isa ring wonderful woman. Ayon sa head writer ng soap na si Suzette Doctolero, hindi ito tulad ng My Husband's Lover na una niyang ginawa. Pero ididirek din ito ni Dominic Zapata at makakasama ni Marian sina Luis Alandy, Mike Tan, TJ Trinidad, Glaiza de Castro, Katrina Halili, Glydel Mercado, Al Tantay at si Ms. Gloria Romero. Sa susunod na buwan na magsisimula ang taping nila nito at after Holy Week naman ang airing. Samantala sina Marian at Dingdong ang first guests sa season six ng The Tim Yap Show at maraming kilig moments sa mag-asawa sa mga tanong ni Tim. After the wedding and honeymoon na ang questions like ano ang feeling ngayong mag-asawa na sila? "Nagugulat pa ako kapag tinatawag akong Mrs. Dantes," sagot ni Marian. "At napapangiti ako sa realization na kasal na nga pala ako kay Dingdong." "Napapatigil naman ako kapag nagpi-fill up ako ng document na pagdating sa civil status, napapangiti ako dahil hindi na nga pala ako single," natatawang sagot ni Dingdong. Nakumusta ni Tim ang ama ni Marian na na-meet niya una sa wedding then sa Boracay. "Promise ni Papa, babalik siya muli sa Pilipinas kapag nalamang preggy na ako. Kung sakali, sa akin unang magkakaapo sina Papa at Mama," sabi ng Primetime Queen ng GMA-7. May pangalan na ba silang nakahanda para sa magiging anak nila? "Since Jose Sixto III ako, hindi pa namin alam kung magiging Jose Sixto IV if boy ang magiging anak namin pero kapag girl, laging magkakaroon iyon ng Maria." Simple lang ang wishes ng mag-asawa. Si Dingdong, ayaw niyang mawawalan ng charge ang cellphone niya kaya lagi siyang may dalang powerbank para lagi niyang nakakausap ang esposa. Gusto ni Marian na laging malinis ang kanilang room hanggang banyo kaya siya ang laging naglilinis nito. Hindi siya nagbubukas ng ilaw habang natutulog pa si Dingdong.</t>
         </is>
       </c>
       <c r="C1076" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Add article cleaning script with comprehensive preprocessing steps and update cleaned Excel files
</commit_message>
<xml_diff>
--- a/HF_cleaned.xlsx
+++ b/HF_cleaned.xlsx
@@ -6882,7 +6882,7 @@
       </c>
       <c r="B257" s="3" t="inlineStr">
         <is>
-          <t>Kabilang sa mga reporma ngayong taon ang mas mabilis at mas maginhawang pakikipagtransaksiyon sa BOC, mas mahusay na koleksiyon ng buwis, at isang pinaigting na kampanya laban sa smuggling. Ang pinakamahalaga sa mga ito ay ang modernisasyon at automation ng mga serbisyo na nakaangkla sa pagpapatupad ng updated e-commerce technology bilang paghahanda sa paglulunsad ng ASEAN Economic Community. Sa Hunyo 2015, ang BOC, sa pamumuno ni Commissioner John Philip P. Sevilla, ay tinatanaw ang katuparan ng mga sumusunod na programa: fully electronic, paperless bureau; single, centralized assessment service; single, centralized valuation database; sale or disposition ng mga produktong inabandona, kinumpiska o isinuko bilang penalty sa loob ng dalawang buwan matapos ibaba ng resolusyon ng legal proceedings; at full electronic record-keeping para sa Customs-bonded na mga warehouse. Magiging katuwang ito ng limang taon na Strategic Plan (2013-2017), na isang action-oriented initiative upang gawing mahusay ang administrasyon ng Customs sa pamamagitan ng goal-setting at resource allocation hanggang 2017. Mayroong open engagement ang BOC sa pribadong seKtor sa pagbabalangkas ng mga polisiya, kung saan ginagawa ang karamihan ng mga aktibidad sa pakikipagkonsulta sa aktibong partisipasyon ng mga partner nito. Ang isang katanggap-tanggap na BOC project ay ang online tracking system ( na inilusad noong Disyembre 2014, kung saan maaaring makita ng mga tatanggap at nagpadala ng mga balikbayan box ang status nito. Laman ng tracker ang listahan ng lahat ng balikbayan box shipment na tangan ng mga lokal na cargo forwarder sa Customs, ang bansang pinanggalingan nito, ang papasukang daungan nito sa Pilipinas, at ang bills of lading na may bilang ng mga shipment.</t>
+          <t>Kabilang sa mga reporma ngayong taon ang mas mabilis at mas maginhawang pakikipagtransaksiyon sa BOC, mas mahusay na koleksiyon ng buwis, at isang pinaigting na kampanya laban sa smuggling. Ang pinakamahalaga sa mga ito ay ang modernisasyon at automation ng mga serbisyo na nakaangkla sa pagpapatupad ng updated e-commerce technology bilang paghahanda sa paglulunsad ng ASEAN Economic Community. Sa Hunyo 2015, ang BOC, sa pamumuno ni Commissioner John Philip P. Sevilla, ay tinatanaw ang katuparan ng mga sumusunod na programa: fully electronic, paperless bureau; single, centralized assessment service; single, centralized valuation database; sale or disposition ng mga produktong inabandona, kinumpiska o isinuko bilang penalty sa loob ng dalawang buwan matapos ibaba ng resolusyon ng legal proceedings; at full electronic record-keeping para sa Customs-bonded na mga warehouse. Magiging katuwang ito ng limang taon na Strategic Plan (2013-2017), na isang action-oriented initiative upang gawing mahusay ang administrasyon ng Customs sa pamamagitan ng goal-setting at resource allocation hanggang 2017. Mayroong open engagement ang BOC sa pribadong seKtor sa pagbabalangkas ng mga polisiya, kung saan ginagawa ang karamihan ng mga aktibidad sa pakikipagkonsulta sa aktibong partisipasyon ng mga partner nito. Ang isang katanggap-tanggap na BOC project ay ang online tracking system ([LINK] na inilusad noong Disyembre 2014, kung saan maaaring makita ng mga tatanggap at nagpadala ng mga balikbayan box ang status nito. Laman ng tracker ang listahan ng lahat ng balikbayan box shipment na tangan ng mga lokal na cargo forwarder sa Customs, ang bansang pinanggalingan nito, ang papasukang daungan nito sa Pilipinas, at ang bills of lading na may bilang ng mga shipment.</t>
         </is>
       </c>
       <c r="C257" s="2" t="inlineStr">
@@ -12132,7 +12132,7 @@
       </c>
       <c r="B467" s="3" t="inlineStr">
         <is>
-          <t>Ibinahagi ni Alden kung gaano kasaya at ka-challenging na makatrabaho ang superstar. "Siya 'yung epitome ng perfect acting, eh. Natural na natural. Alam mo na 'yung mga words na ginagamit niya ay galing sa puso talaga. Sobrang nag-enjoy talaga ako na nakatrabaho ko siya at mas lalong nadagdagan ang self-confidence ko dahil nagkaroon ako ng pagkakataon na makatrabaho ang nag-iisang superstar." Proud siya na kinatawan niya ang bansa sa nasabing international film festival. "It's such a blessing to experience attending this film festival. I was able to meet the stars and directors from different countries at paniguradong isa ito sa highlights ng aking career bilang isang aktor. The experience inspires me to do more and be the best that I can be." Samantala, napansin naman ng isang Vietnamese entertainment website na si Alden at tinawag pa nila itong "Dien vien noi tieng cua" o sa Ingles ay Philippines' Famous Actor.</t>
+          <t>Ibinahagi ni Alden kung gaano kasaya at ka-challenging na makatrabaho ang superstar. "Siya 'yung epitome ng perfect acting, eh. Natural na natural. Alam mo na 'yung mga words na ginagamit niya ay galing sa puso talaga. Sobrang nag-enjoy talaga ako na nakatrabaho ko siya at mas lalong nadagdagan ang self-confidence ko dahil nagkaroon ako ng pagkakataon na makatrabaho ang nag-iisang superstar." Proud siya na kinatawan niya ang bansa sa nasabing international film festival. "It's such a blessing to experience attending this film festival. I was able to meet the stars and directors from different countries at paniguradong isa ito sa highlights ng aking career bilang isang aktor. The experience inspires me to do more and be the best that I can be." Samantala, napansin naman ng isang Vietnamese entertainment website na [LINK] si Alden at tinawag pa nila itong "Dien vien noi tieng cua" o sa Ingles ay Philippines' Famous Actor.</t>
         </is>
       </c>
       <c r="C467" s="2" t="inlineStr">
@@ -16907,7 +16907,7 @@
       </c>
       <c r="B658" s="3" t="inlineStr">
         <is>
-          <t>NAIS itama ng Bandera ang pagkakamali sa isang istorya nito na naipost sa website noong Pebrero 4. Nagpapasalamat ang Bandera kay Sheila Mateo, kamag-anak ng pinaslang na si Boyet San Buenaventura, sa pagtawag sa atensyon sa Bandera ukol sa pagkakamali nito. Si San Buenaventura ang may-ari ng tindahan na pinaslang umano ng bumibili na si Jessie Mark Batugon; at hindi gaya nang napaunang ulat hindi lang Bandera kundi sa iba pang mga news website. (Read more) Narito ang itinamang istorya: PATAY ang isang 37-anyos na lalaki matapos barilin sa kanyang tindahan sa Gumaca, Quezon bago maghatinggabi noong Linggo, Pebrero 3, ayon sa pulisya. Kinilala ni Senior Supt. Osmundo de Guzman, Quezon police director, ang nasawi na Boyet San Buenaventura. Isang police manhunt naman ang inilunsad laban sa suspek na si Jessie Mark Batugon, 19, sa Barangay Progreso. Sa kuwento ng kamag-anak ng biktima na si Sheila Mateo, pumunta si Batugon sa tindahan upang bumili ng noodles. Ang nagbabantay sa tindahan ay ang misis ng nasawi na si Cristina. Nakita umano ng suspek ang biktima na nagtungo sa likuran ng tindahan at doon ay umiihi; pinuntahan ito ng suspek at doon binaril ang biktima sa likod gamit ang .22 kalibreng baril. Binawian ng buhay ang biktima habang dinadala sa San Diego Hospital. Narekober ng mga pulis ang baril, bagamat nakatakas ang suspek. Nanawagan ng hustisya ang mga kamag-anak ng biktima</t>
+          <t>NAIS itama ng Bandera ang pagkakamali sa isang istorya nito na naipost sa website noong Pebrero 4. Nagpapasalamat ang Bandera kay Sheila Mateo, kamag-anak ng pinaslang na si Boyet San Buenaventura, sa pagtawag sa atensyon sa Bandera ukol sa pagkakamali nito. Si San Buenaventura ang may-ari ng tindahan na pinaslang umano ng bumibili na si Jessie Mark Batugon; at hindi gaya nang napaunang ulat hindi lang Bandera kundi sa iba pang mga news website. (Read more) [LINK] Narito ang itinamang istorya: PATAY ang isang 37-anyos na lalaki matapos barilin sa kanyang tindahan sa Gumaca, Quezon bago maghatinggabi noong Linggo, Pebrero 3, ayon sa pulisya. Kinilala ni Senior Supt. Osmundo de Guzman, Quezon police director, ang nasawi na Boyet San Buenaventura. Isang police manhunt naman ang inilunsad laban sa suspek na si Jessie Mark Batugon, 19, sa Barangay Progreso. Sa kuwento ng kamag-anak ng biktima na si Sheila Mateo, pumunta si Batugon sa tindahan upang bumili ng noodles. Ang nagbabantay sa tindahan ay ang misis ng nasawi na si Cristina. Nakita umano ng suspek ang biktima na nagtungo sa likuran ng tindahan at doon ay umiihi; pinuntahan ito ng suspek at doon binaril ang biktima sa likod gamit ang .22 kalibreng baril. Binawian ng buhay ang biktima habang dinadala sa San Diego Hospital. Narekober ng mga pulis ang baril, bagamat nakatakas ang suspek. Nanawagan ng hustisya ang mga kamag-anak ng biktima</t>
         </is>
       </c>
       <c r="C658" s="2" t="inlineStr">
@@ -21157,7 +21157,7 @@
       </c>
       <c r="B828" s="5" t="inlineStr">
         <is>
-          <t>Gayunman, hinimok ng PHLPost ang publiko na bumibili online na isumite ang kanilang mga stamp order sa Pinoy eMall site upang makabili sa aktuwal na presyo. "Upang protektahan ang interes ng publiko, hinihikayat namin ang lahat na magkaroon ng bahagi sa Pope Francis memorabilia sa pamamagitan ng mga selyo na mabibili online sa pamamagitan ng PHLPost web portal, at face value," sabi ni Postmaster General Josie Dela Cruz. Ito ang naging panawagan ng PHLPost kasunod ng mga ulat na ibinebenta sa black market ang mga kopya ng nasabing commemorative stamp nang doble sa aktuwal na presyo nito. Upang makabili ng mga stamp, mag-log on sa at i-click ang Pinoy eMall na magbubukas sa website na Pinoy e-Mall.</t>
+          <t>Gayunman, hinimok ng PHLPost ang publiko na bumibili online na isumite ang kanilang mga stamp order sa Pinoy eMall site upang makabili sa aktuwal na presyo. "Upang protektahan ang interes ng publiko, hinihikayat namin ang lahat na magkaroon ng bahagi sa Pope Francis memorabilia sa pamamagitan ng mga selyo na mabibili online sa pamamagitan ng PHLPost web portal, at face value," sabi ni Postmaster General Josie Dela Cruz. Ito ang naging panawagan ng PHLPost kasunod ng mga ulat na ibinebenta sa black market ang mga kopya ng nasabing commemorative stamp nang doble sa aktuwal na presyo nito. Upang makabili ng mga stamp, mag-log on sa [LINK] at i-click ang Pinoy eMall na magbubukas sa website na Pinoy e-Mall.</t>
         </is>
       </c>
       <c r="C828" s="4" t="inlineStr">

</xml_diff>